<commit_message>
make econ losses intensity based
</commit_message>
<xml_diff>
--- a/data/raw/Economic damages source review.xlsx
+++ b/data/raw/Economic damages source review.xlsx
@@ -37,7 +37,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment authorId="0" ref="I8">
+    <comment authorId="0" ref="J8">
       <text>
         <t xml:space="preserve">Should also interpolate
 	-Sebastian Barungi Rugunda Quaade</t>
@@ -49,13 +49,13 @@
 	-Sebastian Barungi Rugunda Quaade</t>
       </text>
     </comment>
-    <comment authorId="0" ref="G3">
+    <comment authorId="0" ref="H3">
       <text>
         <t xml:space="preserve">This is a guess since they don't document the reference year for their valuations
 	-Sebastian Barungi Rugunda Quaade</t>
       </text>
     </comment>
-    <comment authorId="0" ref="I6">
+    <comment authorId="0" ref="J6">
       <text>
         <t xml:space="preserve">Should actually interpolate to get this, but approximately right for now
 	-Sebastian Barungi Rugunda Quaade</t>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="75">
   <si>
     <r>
       <rPr/>
@@ -246,6 +246,9 @@
     <t>Mortality (SMU)</t>
   </si>
   <si>
+    <t>Intensity (SMU)</t>
+  </si>
+  <si>
     <t>GDP loss year</t>
   </si>
   <si>
@@ -259,6 +262,9 @@
   </si>
   <si>
     <t>Fraction GDP losses</t>
+  </si>
+  <si>
+    <t>Annual fraction GPD losses</t>
   </si>
   <si>
     <t>Other notes</t>
@@ -547,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -603,9 +609,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
@@ -730,7 +733,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Updated numbers'!$K$1:$K$9</c:f>
+              <c:f>'Updated numbers'!$L$1:$L$9</c:f>
               <c:numCache/>
             </c:numRef>
           </c:yVal>
@@ -743,11 +746,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1646809150"/>
-        <c:axId val="1108436848"/>
+        <c:axId val="1543745231"/>
+        <c:axId val="303530121"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1646809150"/>
+        <c:axId val="1543745231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -822,10 +825,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1108436848"/>
+        <c:crossAx val="303530121"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1108436848"/>
+        <c:axId val="303530121"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.3"/>
@@ -901,7 +904,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1646809150"/>
+        <c:crossAx val="1543745231"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -939,7 +942,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>161925</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
@@ -1449,14 +1452,14 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="6" max="6" width="16.13"/>
-    <col customWidth="1" min="7" max="8" width="21.63"/>
-    <col customWidth="1" min="9" max="9" width="18.75"/>
-    <col customWidth="1" min="10" max="10" width="18.38"/>
-    <col customWidth="1" min="11" max="11" width="16.5"/>
-    <col customWidth="1" min="12" max="12" width="38.5"/>
-    <col customWidth="1" min="13" max="13" width="18.88"/>
-    <col customWidth="1" min="14" max="14" width="33.0"/>
-    <col customWidth="1" min="15" max="15" width="30.13"/>
+    <col customWidth="1" min="7" max="9" width="21.63"/>
+    <col customWidth="1" min="10" max="10" width="18.75"/>
+    <col customWidth="1" min="11" max="11" width="18.38"/>
+    <col customWidth="1" min="12" max="13" width="16.5"/>
+    <col customWidth="1" min="14" max="14" width="38.5"/>
+    <col customWidth="1" min="15" max="15" width="18.88"/>
+    <col customWidth="1" min="16" max="16" width="33.0"/>
+    <col customWidth="1" min="17" max="17" width="30.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1494,19 +1497,23 @@
         <v>37</v>
       </c>
       <c r="L1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
+      <c r="Q1" s="13" t="s">
+        <v>40</v>
+      </c>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
       <c r="T1" s="4"/>
@@ -1520,6 +1527,8 @@
       <c r="AB1" s="4"/>
       <c r="AC1" s="4"/>
       <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
@@ -1539,35 +1548,43 @@
       <c r="F2" s="15">
         <v>5.59913E-5</v>
       </c>
-      <c r="G2" s="6">
-        <v>2015.0</v>
+      <c r="G2" s="15">
+        <f t="shared" ref="G2:G6" si="2">F2/D2</f>
+        <v>0.00001866376667</v>
       </c>
       <c r="H2" s="6">
         <v>2015.0</v>
       </c>
       <c r="I2" s="6">
+        <v>2015.0</v>
+      </c>
+      <c r="J2" s="6">
         <f>7*1000000000</f>
         <v>7000000000</v>
       </c>
-      <c r="J2" s="6">
-        <f>I2*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H2,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K2" s="6">
+        <f>J2*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I2,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>8645147679</v>
       </c>
-      <c r="K2" s="16">
-        <f>J2/VLOOKUP(G2,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
+      <c r="L2" s="16">
+        <f>K2/VLOOKUP(H2,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
         <v>0.0000635021097</v>
       </c>
-      <c r="L2" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="16">
+        <f t="shared" ref="M2:M6" si="3">L2/D2</f>
+        <v>0.0000211673699</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="O2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>41</v>
+      <c r="P2" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" s="13" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -1589,33 +1606,41 @@
         <v>0.00116592761933782</v>
       </c>
       <c r="G3" s="6">
-        <v>2005.0</v>
+        <f t="shared" si="2"/>
+        <v>0.0005829638097</v>
       </c>
       <c r="H3" s="6">
         <v>2005.0</v>
       </c>
       <c r="I3" s="6">
+        <v>2005.0</v>
+      </c>
+      <c r="J3" s="6">
         <f>11.8*1000000000</f>
         <v>11800000000</v>
       </c>
-      <c r="J3" s="6">
-        <f>I3*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H3,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K3" s="6">
+        <f>J3*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I3,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>17684895033</v>
       </c>
-      <c r="K3" s="16">
-        <f>J3/VLOOKUP(G3,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
+      <c r="L3" s="16">
+        <f>K3/VLOOKUP(H3,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
         <v>0.0001808169642</v>
       </c>
-      <c r="L3" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>43</v>
+      <c r="M3" s="16">
+        <f t="shared" si="3"/>
+        <v>0.00009040848211</v>
       </c>
       <c r="N3" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="O3" s="13"/>
+      <c r="O3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="13"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
@@ -1638,33 +1663,41 @@
         <v>0.0157</v>
       </c>
       <c r="G4" s="6">
-        <v>2014.0</v>
+        <f t="shared" si="2"/>
+        <v>0.003925</v>
       </c>
       <c r="H4" s="6">
         <v>2014.0</v>
       </c>
       <c r="I4" s="6">
+        <v>2014.0</v>
+      </c>
+      <c r="J4" s="6">
         <f>15.67*3*1000000000</f>
         <v>47010000000</v>
       </c>
-      <c r="J4" s="6">
-        <f>I4*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H4,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K4" s="6">
+        <f>J4*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I4,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>58131926489</v>
       </c>
-      <c r="K4" s="16">
-        <f>J4/VLOOKUP(G4,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
+      <c r="L4" s="16">
+        <f>K4/VLOOKUP(H4,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
         <v>0.0004385431439</v>
       </c>
-      <c r="L4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="M4" s="10" t="s">
+      <c r="M4" s="16">
+        <f t="shared" si="3"/>
+        <v>0.000109635786</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="O4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="O4" s="14"/>
+      <c r="P4" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q4" s="14"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
@@ -1687,33 +1720,41 @@
         <v>4.59</v>
       </c>
       <c r="G5" s="6">
-        <v>2019.0</v>
+        <f t="shared" si="2"/>
+        <v>0.918</v>
       </c>
       <c r="H5" s="6">
         <v>2019.0</v>
       </c>
       <c r="I5" s="6">
+        <v>2019.0</v>
+      </c>
+      <c r="J5" s="6">
         <f>13800000000000</f>
         <v>13800000000000</v>
       </c>
-      <c r="J5" s="6">
-        <f>I5*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H5,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K5" s="6">
+        <f>J5*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I5,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>15796871333594</v>
       </c>
-      <c r="K5" s="16">
-        <f>J5/VLOOKUP(G5,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
+      <c r="L5" s="16">
+        <f>K5/VLOOKUP(H5,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
         <v>0.1009765141</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="M5" s="16">
+        <f t="shared" si="3"/>
+        <v>0.02019530282</v>
+      </c>
+      <c r="N5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="O5" s="14"/>
+      <c r="O5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q5" s="14"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
@@ -1736,37 +1777,45 @@
         <v>171.0</v>
       </c>
       <c r="G6" s="6">
+        <f t="shared" si="2"/>
+        <v>57</v>
+      </c>
+      <c r="H6" s="6">
         <v>1917.0</v>
       </c>
-      <c r="H6" s="6">
+      <c r="I6" s="6">
         <f>Constants!$B$1</f>
         <v>2022</v>
       </c>
-      <c r="I6" s="15">
-        <f>K6*VLOOKUP(G6, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
+      <c r="J6" s="15">
+        <f>L6*VLOOKUP(H6, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
         <v>300223500612</v>
       </c>
-      <c r="J6" s="15">
-        <f>I6*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H6,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K6" s="15">
+        <f>J6*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I6,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>300223500612</v>
       </c>
-      <c r="K6" s="20">
+      <c r="L6" s="20">
         <v>0.06</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="M6" s="16">
+        <f t="shared" si="3"/>
+        <v>0.02</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="O6" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="N6" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="O6" s="14"/>
+      <c r="P6" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q6" s="14"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
@@ -1777,14 +1826,16 @@
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
       <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" s="8">
         <v>1968.0</v>
@@ -1801,62 +1852,72 @@
         <v>2.82</v>
       </c>
       <c r="G8" s="6">
+        <f>F8/D8</f>
+        <v>0.94</v>
+      </c>
+      <c r="H8" s="6">
         <f>'Global GDP over time'!$I$4</f>
         <v>2017</v>
       </c>
-      <c r="H8" s="6">
+      <c r="I8" s="6">
         <f>Constants!$B$1</f>
         <v>2022</v>
       </c>
-      <c r="I8" s="15">
-        <f>K8*VLOOKUP(G8, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
+      <c r="J8" s="15">
+        <f>L8*VLOOKUP(H8, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
         <v>3525297429621</v>
       </c>
-      <c r="J8" s="15">
-        <f>I8*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(H8,'US CPI'!$A$2:$B$114,2,FALSE))</f>
+      <c r="K8" s="15">
+        <f>J8*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I8,'US CPI'!$A$2:$B$114,2,FALSE))</f>
         <v>3525297429621</v>
       </c>
-      <c r="K8" s="21">
+      <c r="L8" s="20">
         <v>0.024</v>
       </c>
-      <c r="L8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="M8" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
+      <c r="M8" s="16">
+        <f>L8/D8</f>
+        <v>0.008</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="O8" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
+      <c r="M9" s="16"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId2" ref="L2"/>
-    <hyperlink r:id="rId3" ref="M3"/>
-    <hyperlink r:id="rId4" ref="M4"/>
-    <hyperlink r:id="rId5" ref="L5"/>
-    <hyperlink r:id="rId6" ref="M5"/>
-    <hyperlink r:id="rId7" ref="M6"/>
-    <hyperlink r:id="rId8" ref="N6"/>
-    <hyperlink r:id="rId9" ref="M8"/>
+    <hyperlink r:id="rId2" ref="N2"/>
+    <hyperlink r:id="rId3" ref="O3"/>
+    <hyperlink r:id="rId4" ref="O4"/>
+    <hyperlink r:id="rId5" ref="N5"/>
+    <hyperlink r:id="rId6" ref="O5"/>
+    <hyperlink r:id="rId7" ref="O6"/>
+    <hyperlink r:id="rId8" ref="P6"/>
+    <hyperlink r:id="rId9" ref="O8"/>
   </hyperlinks>
   <drawing r:id="rId10"/>
   <legacyDrawing r:id="rId11"/>
@@ -1875,900 +1936,900 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="B1" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="C1" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="D1" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="E1" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="24" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" s="27">
+      <c r="A2" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="26">
         <v>1.0</v>
       </c>
-      <c r="D2" s="28">
+      <c r="D2" s="27">
         <v>2.13E11</v>
       </c>
-      <c r="E2" s="29">
+      <c r="E2" s="28">
         <f>D2*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>254365973072</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="H2" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="B3" s="22" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="27">
+      <c r="C3" s="26">
         <v>1000.0</v>
       </c>
-      <c r="D3" s="28">
+      <c r="D3" s="27">
         <v>2.46E11</v>
       </c>
-      <c r="E3" s="29">
+      <c r="E3" s="28">
         <f>D3*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>293774785802</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="27">
+      <c r="A4" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="26">
         <v>1500.0</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="27">
         <v>5.03E11</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="28">
         <f>D4*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>600685842513</v>
       </c>
-      <c r="H4" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="I4" s="25">
+      <c r="H4" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="24">
         <v>2017.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="27">
+      <c r="A5" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="26">
         <v>1600.0</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="27">
         <v>6.71E11</v>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="28">
         <f>D5*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>801312525500</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="27">
+      <c r="A6" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="26">
         <v>1700.0</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="27">
         <v>7.52E11</v>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="28">
         <f>D6*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>898043247654</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="27">
+      <c r="A7" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="26">
         <v>1820.0</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="27">
         <v>1.4E12</v>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="28">
         <f>D7*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>1671889024888</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="27">
+      <c r="A8" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="26">
         <v>1850.0</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="27">
         <v>1.85E12</v>
       </c>
-      <c r="E8" s="29">
+      <c r="E8" s="28">
         <f>D8*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>2209281925745</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="27">
+      <c r="A9" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="26">
         <v>1870.0</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="27">
         <v>2.35E12</v>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="28">
         <f>D9*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>2806385148919</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="27">
+      <c r="A10" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="26">
         <v>1900.0</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="27">
         <v>4.19E12</v>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="28">
         <f>D10*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>5003725010200</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="27">
+      <c r="A11" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="26">
         <v>1920.0</v>
       </c>
-      <c r="D11" s="28">
+      <c r="D11" s="27">
         <v>5.77E12</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="28">
         <f>D11*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>6890571195430</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="27">
+      <c r="A12" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="26">
         <v>1940.0</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="27">
         <v>9.14E12</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="28">
         <f>D12*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>10915046919625</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="27">
+      <c r="A13" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="26">
         <v>1950.0</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="27">
         <v>1.01E13</v>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="28">
         <f>D13*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>12061485108119</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="27">
+      <c r="A14" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="26">
         <v>1960.0</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="27">
         <v>1.59E13</v>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="28">
         <f>D14*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>18987882496940</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="27">
+      <c r="A15" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="26">
         <v>1970.0</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="27">
         <v>2.62E13</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="28">
         <f>D15*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>31288208894329</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="27">
+      <c r="A16" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="26">
         <v>1980.0</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="27">
         <v>3.82E13</v>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="28">
         <f>D16*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>45618686250510</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="27">
+      <c r="A17" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="26">
         <v>1990.0</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="27">
         <v>5.14E13</v>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="28">
         <f>D17*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>61382211342309</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="27">
+      <c r="A18" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="26">
         <v>1991.0</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="27">
         <v>5.21E13</v>
       </c>
-      <c r="E18" s="29">
+      <c r="E18" s="28">
         <f>D18*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>62218155854753</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="27">
+      <c r="A19" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="26">
         <v>1992.0</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="27">
         <v>5.29E13</v>
       </c>
-      <c r="E19" s="29">
+      <c r="E19" s="28">
         <f>D19*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>63173521011832</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="27">
+      <c r="A20" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="26">
         <v>1993.0</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="27">
         <v>5.38E13</v>
       </c>
-      <c r="E20" s="29">
+      <c r="E20" s="28">
         <f>D20*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>64248306813546</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="27">
+      <c r="A21" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="26">
         <v>1994.0</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="27">
         <v>5.54E13</v>
       </c>
-      <c r="E21" s="29">
+      <c r="E21" s="28">
         <f>D21*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>66159037127703</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C22" s="27">
+      <c r="A22" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="26">
         <v>1995.0</v>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="27">
         <v>5.71E13</v>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="28">
         <f>D22*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>68189188086495</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="27">
+      <c r="A23" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="26">
         <v>1996.0</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="27">
         <v>5.92E13</v>
       </c>
-      <c r="E23" s="29">
+      <c r="E23" s="28">
         <f>D23*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>70697021623827</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="27">
+      <c r="A24" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="26">
         <v>1997.0</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="27">
         <v>6.16E13</v>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="28">
         <f>D24*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>73563117095063</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="27">
+      <c r="A25" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="26">
         <v>1998.0</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="27">
         <v>6.31E13</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="28">
         <f>D25*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>75354426764586</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C26" s="27">
+      <c r="A26" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="26">
         <v>1999.0</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="27">
         <v>6.53E13</v>
       </c>
-      <c r="E26" s="29">
+      <c r="E26" s="28">
         <f>D26*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>77981680946552</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="27">
+      <c r="A27" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="26">
         <v>2000.0</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="27">
         <v>6.84E13</v>
       </c>
-      <c r="E27" s="29">
+      <c r="E27" s="28">
         <f>D27*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>81683720930233</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B28" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="27">
+      <c r="A28" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="26">
         <v>2001.0</v>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="27">
         <v>7.0E13</v>
       </c>
-      <c r="E28" s="29">
+      <c r="E28" s="28">
         <f>D28*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>83594451244390</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="27">
+      <c r="A29" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="26">
         <v>2002.0</v>
       </c>
-      <c r="D29" s="28">
+      <c r="D29" s="27">
         <v>7.19E13</v>
       </c>
-      <c r="E29" s="29">
+      <c r="E29" s="28">
         <f>D29*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>85863443492452</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="27">
+      <c r="A30" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="26">
         <v>2003.0</v>
       </c>
-      <c r="D30" s="28">
+      <c r="D30" s="27">
         <v>7.46E13</v>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="28">
         <f>D30*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>89087800897593</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="27">
+      <c r="A31" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="26">
         <v>2004.0</v>
       </c>
-      <c r="D31" s="28">
+      <c r="D31" s="27">
         <v>7.83E13</v>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="28">
         <f>D31*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>93506364749082</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="27">
+      <c r="A32" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="26">
         <v>2005.0</v>
       </c>
-      <c r="D32" s="28">
+      <c r="D32" s="27">
         <v>8.19E13</v>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="28">
         <f>D32*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>97805507955936</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="27">
+      <c r="A33" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="26">
         <v>2006.0</v>
       </c>
-      <c r="D33" s="28">
+      <c r="D33" s="27">
         <v>8.61E13</v>
       </c>
-      <c r="E33" s="29">
+      <c r="E33" s="28">
         <f>D33*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>102821175030600</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B34" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C34" s="27">
+      <c r="A34" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="26">
         <v>2007.0</v>
       </c>
-      <c r="D34" s="28">
+      <c r="D34" s="27">
         <v>9.05E13</v>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="28">
         <f>D34*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>108075683394533</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C35" s="27">
+      <c r="A35" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="26">
         <v>2008.0</v>
       </c>
-      <c r="D35" s="28">
+      <c r="D35" s="27">
         <v>9.29E13</v>
       </c>
-      <c r="E35" s="29">
+      <c r="E35" s="28">
         <f>D35*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>110941778865769</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B36" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="27">
+      <c r="A36" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="26">
         <v>2009.0</v>
       </c>
-      <c r="D36" s="28">
+      <c r="D36" s="27">
         <v>9.22E13</v>
       </c>
-      <c r="E36" s="29">
+      <c r="E36" s="28">
         <f>D36*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>110105834353325</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="27">
+      <c r="A37" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" s="26">
         <v>2010.0</v>
       </c>
-      <c r="D37" s="28">
+      <c r="D37" s="27">
         <v>9.69E13</v>
       </c>
-      <c r="E37" s="29">
+      <c r="E37" s="28">
         <f>D37*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>115718604651163</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B38" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="27">
+      <c r="A38" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="26">
         <v>2011.0</v>
       </c>
-      <c r="D38" s="28">
+      <c r="D38" s="27">
         <v>1.01E14</v>
       </c>
-      <c r="E38" s="29">
+      <c r="E38" s="28">
         <f>D38*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>120614851081191</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B39" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C39" s="27">
+      <c r="A39" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="26">
         <v>2012.0</v>
       </c>
-      <c r="D39" s="28">
+      <c r="D39" s="27">
         <v>1.04E14</v>
       </c>
-      <c r="E39" s="29">
+      <c r="E39" s="28">
         <f>D39*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>124197470420237</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B40" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C40" s="27">
+      <c r="A40" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C40" s="26">
         <v>2013.0</v>
       </c>
-      <c r="D40" s="28">
+      <c r="D40" s="27">
         <v>1.07E14</v>
       </c>
-      <c r="E40" s="29">
+      <c r="E40" s="28">
         <f>D40*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>127780089759282</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B41" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C41" s="27">
+      <c r="A41" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="26">
         <v>2014.0</v>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="27">
         <v>1.11E14</v>
       </c>
-      <c r="E41" s="29">
+      <c r="E41" s="28">
         <f>D41*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>132556915544676</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B42" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C42" s="27">
+      <c r="A42" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B42" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="26">
         <v>2015.0</v>
       </c>
-      <c r="D42" s="28">
+      <c r="D42" s="27">
         <v>1.14E14</v>
       </c>
-      <c r="E42" s="29">
+      <c r="E42" s="28">
         <f>D42*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>136139534883721</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B43" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C43" s="27">
+      <c r="A43" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C43" s="26">
         <v>2016.0</v>
       </c>
-      <c r="D43" s="28">
+      <c r="D43" s="27">
         <v>1.18E14</v>
       </c>
-      <c r="E43" s="29">
+      <c r="E43" s="28">
         <f>D43*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>140916360669115</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C44" s="27">
+      <c r="A44" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B44" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" s="26">
         <v>2017.0</v>
       </c>
-      <c r="D44" s="28">
+      <c r="D44" s="27">
         <v>1.23E14</v>
       </c>
-      <c r="E44" s="29">
+      <c r="E44" s="28">
         <f>D44*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>146887392900857</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B45" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C45" s="27">
+      <c r="A45" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C45" s="26">
         <v>2018.0</v>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="27">
         <v>1.27E14</v>
       </c>
-      <c r="E45" s="29">
+      <c r="E45" s="28">
         <f>D45*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>151664218686251</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B46" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C46" s="27">
+      <c r="A46" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="26">
         <v>2019.0</v>
       </c>
-      <c r="D46" s="28">
+      <c r="D46" s="27">
         <v>1.31E14</v>
       </c>
-      <c r="E46" s="29">
+      <c r="E46" s="28">
         <f>D46*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>156441044471644</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B47" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C47" s="27">
+      <c r="A47" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C47" s="26">
         <v>2020.0</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="27">
         <v>1.27E14</v>
       </c>
-      <c r="E47" s="29">
+      <c r="E47" s="28">
         <f>D47*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>151664218686251</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B48" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C48" s="27">
+      <c r="A48" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B48" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" s="26">
         <v>2021.0</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="27">
         <v>1.35E14</v>
       </c>
-      <c r="E48" s="29">
+      <c r="E48" s="28">
         <f>D48*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>161217870257038</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B49" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C49" s="27">
+      <c r="A49" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C49" s="26">
         <v>2022.0</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="27">
         <v>1.39E14</v>
       </c>
-      <c r="E49" s="29">
+      <c r="E49" s="28">
         <f>D49*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
         <v>165994696042432</v>
       </c>
@@ -2789,10 +2850,10 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="25">
+      <c r="A1" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="24">
         <v>2022.0</v>
       </c>
     </row>
@@ -2813,2163 +2874,2163 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>59</v>
+      <c r="A1" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="25" t="s">
+      <c r="A2" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="C2" s="24" t="s">
         <v>71</v>
       </c>
+      <c r="E2" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="29" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="25">
+      <c r="A3" s="24">
         <v>1913.0</v>
       </c>
-      <c r="B3" s="25">
+      <c r="B3" s="24">
         <v>9.9</v>
       </c>
-      <c r="E3" s="32">
+      <c r="E3" s="31">
         <f t="shared" ref="E3:E114" si="1">A3</f>
         <v>1913</v>
       </c>
-      <c r="F3" s="32">
+      <c r="F3" s="31">
         <f t="shared" ref="F3:F114" si="2">VLOOKUP(E3,$A$3:$B$114,2,FALSE)/VLOOKUP($J$3,$A$3:$B$114,2,FALSE)</f>
         <v>0.03382302699</v>
       </c>
-      <c r="I3" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="J3" s="25">
+      <c r="I3" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="J3" s="24">
         <v>2022.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25">
+      <c r="A4" s="24">
         <v>1914.0</v>
       </c>
-      <c r="B4" s="25">
+      <c r="B4" s="24">
         <v>10.0</v>
       </c>
-      <c r="C4" s="33">
+      <c r="C4" s="32">
         <v>0.013</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="31">
         <f t="shared" si="1"/>
         <v>1914</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="31">
         <f t="shared" si="2"/>
         <v>0.03416467373</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25">
+      <c r="A5" s="24">
         <v>1915.0</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="24">
         <v>10.1</v>
       </c>
-      <c r="C5" s="33">
+      <c r="C5" s="32">
         <v>0.009</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="31">
         <f t="shared" si="1"/>
         <v>1915</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="31">
         <f t="shared" si="2"/>
         <v>0.03450632046</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25">
+      <c r="A6" s="24">
         <v>1916.0</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="24">
         <v>10.9</v>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="32">
         <v>0.077</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="31">
         <f t="shared" si="1"/>
         <v>1916</v>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="31">
         <f t="shared" si="2"/>
         <v>0.03723949436</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25">
+      <c r="A7" s="24">
         <v>1917.0</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="24">
         <v>12.8</v>
       </c>
-      <c r="C7" s="33">
+      <c r="C7" s="32">
         <v>0.178</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="31">
         <f t="shared" si="1"/>
         <v>1917</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="31">
         <f t="shared" si="2"/>
         <v>0.04373078237</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25">
+      <c r="A8" s="24">
         <v>1918.0</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="24">
         <v>15.0</v>
       </c>
-      <c r="C8" s="33">
+      <c r="C8" s="32">
         <v>0.173</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="31">
         <f t="shared" si="1"/>
         <v>1918</v>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="31">
         <f t="shared" si="2"/>
         <v>0.05124701059</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25">
+      <c r="A9" s="24">
         <v>1919.0</v>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="24">
         <v>17.3</v>
       </c>
-      <c r="C9" s="33">
+      <c r="C9" s="32">
         <v>0.152</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="31">
         <f t="shared" si="1"/>
         <v>1919</v>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="31">
         <f t="shared" si="2"/>
         <v>0.05910488555</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25">
+      <c r="A10" s="24">
         <v>1920.0</v>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="24">
         <v>20.0</v>
       </c>
-      <c r="C10" s="33">
+      <c r="C10" s="32">
         <v>0.156</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="31">
         <f t="shared" si="1"/>
         <v>1920</v>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="31">
         <f t="shared" si="2"/>
         <v>0.06832934745</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25">
+      <c r="A11" s="24">
         <v>1921.0</v>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="24">
         <v>17.9</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="32">
         <v>-0.109</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="31">
         <f t="shared" si="1"/>
         <v>1921</v>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="31">
         <f t="shared" si="2"/>
         <v>0.06115476597</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25">
+      <c r="A12" s="24">
         <v>1922.0</v>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="24">
         <v>16.8</v>
       </c>
-      <c r="C12" s="33">
+      <c r="C12" s="32">
         <v>-0.062</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="31">
         <f t="shared" si="1"/>
         <v>1922</v>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="31">
         <f t="shared" si="2"/>
         <v>0.05739665186</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25">
+      <c r="A13" s="24">
         <v>1923.0</v>
       </c>
-      <c r="B13" s="25">
+      <c r="B13" s="24">
         <v>17.1</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="32">
         <v>0.018</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="31">
         <f t="shared" si="1"/>
         <v>1923</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="31">
         <f t="shared" si="2"/>
         <v>0.05842159207</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25">
+      <c r="A14" s="24">
         <v>1924.0</v>
       </c>
-      <c r="B14" s="25">
+      <c r="B14" s="24">
         <v>17.1</v>
       </c>
-      <c r="C14" s="33">
+      <c r="C14" s="32">
         <v>0.004</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="31">
         <f t="shared" si="1"/>
         <v>1924</v>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="31">
         <f t="shared" si="2"/>
         <v>0.05842159207</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25">
+      <c r="A15" s="24">
         <v>1925.0</v>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="24">
         <v>17.5</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <v>0.024</v>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="31">
         <f t="shared" si="1"/>
         <v>1925</v>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="31">
         <f t="shared" si="2"/>
         <v>0.05978817902</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25">
+      <c r="A16" s="24">
         <v>1926.0</v>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="24">
         <v>17.7</v>
       </c>
-      <c r="C16" s="33">
+      <c r="C16" s="32">
         <v>0.009</v>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="31">
         <f t="shared" si="1"/>
         <v>1926</v>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="31">
         <f t="shared" si="2"/>
         <v>0.0604714725</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25">
+      <c r="A17" s="24">
         <v>1927.0</v>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="24">
         <v>17.4</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="32">
         <v>-0.019</v>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="31">
         <f t="shared" si="1"/>
         <v>1927</v>
       </c>
-      <c r="F17" s="32">
+      <c r="F17" s="31">
         <f t="shared" si="2"/>
         <v>0.05944653229</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25">
+      <c r="A18" s="24">
         <v>1928.0</v>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="24">
         <v>17.2</v>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="32">
         <v>-0.012</v>
       </c>
-      <c r="E18" s="32">
+      <c r="E18" s="31">
         <f t="shared" si="1"/>
         <v>1928</v>
       </c>
-      <c r="F18" s="32">
+      <c r="F18" s="31">
         <f t="shared" si="2"/>
         <v>0.05876323881</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25">
+      <c r="A19" s="24">
         <v>1929.0</v>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="24">
         <v>17.2</v>
       </c>
-      <c r="C19" s="33">
+      <c r="C19" s="32">
         <v>0.0</v>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="31">
         <f t="shared" si="1"/>
         <v>1929</v>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="31">
         <f t="shared" si="2"/>
         <v>0.05876323881</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25">
+      <c r="A20" s="24">
         <v>1930.0</v>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="24">
         <v>16.7</v>
       </c>
-      <c r="C20" s="33">
+      <c r="C20" s="32">
         <v>-0.027</v>
       </c>
-      <c r="E20" s="32">
+      <c r="E20" s="31">
         <f t="shared" si="1"/>
         <v>1930</v>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="31">
         <f t="shared" si="2"/>
         <v>0.05705500512</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25">
+      <c r="A21" s="24">
         <v>1931.0</v>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="24">
         <v>15.2</v>
       </c>
-      <c r="C21" s="33">
+      <c r="C21" s="32">
         <v>-0.089</v>
       </c>
-      <c r="E21" s="32">
+      <c r="E21" s="31">
         <f t="shared" si="1"/>
         <v>1931</v>
       </c>
-      <c r="F21" s="32">
+      <c r="F21" s="31">
         <f t="shared" si="2"/>
         <v>0.05193030407</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25">
+      <c r="A22" s="24">
         <v>1932.0</v>
       </c>
-      <c r="B22" s="25">
+      <c r="B22" s="24">
         <v>13.6</v>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="32">
         <v>-0.103</v>
       </c>
-      <c r="E22" s="32">
+      <c r="E22" s="31">
         <f t="shared" si="1"/>
         <v>1932</v>
       </c>
-      <c r="F22" s="32">
+      <c r="F22" s="31">
         <f t="shared" si="2"/>
         <v>0.04646395627</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25">
+      <c r="A23" s="24">
         <v>1933.0</v>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="24">
         <v>12.9</v>
       </c>
-      <c r="C23" s="33">
+      <c r="C23" s="32">
         <v>-0.052</v>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="31">
         <f t="shared" si="1"/>
         <v>1933</v>
       </c>
-      <c r="F23" s="32">
+      <c r="F23" s="31">
         <f t="shared" si="2"/>
         <v>0.04407242911</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25">
+      <c r="A24" s="24">
         <v>1934.0</v>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="24">
         <v>13.4</v>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="32">
         <v>0.035</v>
       </c>
-      <c r="E24" s="32">
+      <c r="E24" s="31">
         <f t="shared" si="1"/>
         <v>1934</v>
       </c>
-      <c r="F24" s="32">
+      <c r="F24" s="31">
         <f t="shared" si="2"/>
         <v>0.04578066279</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25">
+      <c r="A25" s="24">
         <v>1935.0</v>
       </c>
-      <c r="B25" s="25">
+      <c r="B25" s="24">
         <v>13.7</v>
       </c>
-      <c r="C25" s="33">
+      <c r="C25" s="32">
         <v>0.026</v>
       </c>
-      <c r="E25" s="32">
+      <c r="E25" s="31">
         <f t="shared" si="1"/>
         <v>1935</v>
       </c>
-      <c r="F25" s="32">
+      <c r="F25" s="31">
         <f t="shared" si="2"/>
         <v>0.04680560301</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25">
+      <c r="A26" s="24">
         <v>1936.0</v>
       </c>
-      <c r="B26" s="25">
+      <c r="B26" s="24">
         <v>13.9</v>
       </c>
-      <c r="C26" s="33">
+      <c r="C26" s="32">
         <v>0.01</v>
       </c>
-      <c r="E26" s="32">
+      <c r="E26" s="31">
         <f t="shared" si="1"/>
         <v>1936</v>
       </c>
-      <c r="F26" s="32">
+      <c r="F26" s="31">
         <f t="shared" si="2"/>
         <v>0.04748889648</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="25">
+      <c r="A27" s="24">
         <v>1937.0</v>
       </c>
-      <c r="B27" s="25">
+      <c r="B27" s="24">
         <v>14.4</v>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="32">
         <v>0.037</v>
       </c>
-      <c r="E27" s="32">
+      <c r="E27" s="31">
         <f t="shared" si="1"/>
         <v>1937</v>
       </c>
-      <c r="F27" s="32">
+      <c r="F27" s="31">
         <f t="shared" si="2"/>
         <v>0.04919713017</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="25">
+      <c r="A28" s="24">
         <v>1938.0</v>
       </c>
-      <c r="B28" s="25">
+      <c r="B28" s="24">
         <v>14.1</v>
       </c>
-      <c r="C28" s="33">
+      <c r="C28" s="32">
         <v>-0.02</v>
       </c>
-      <c r="E28" s="32">
+      <c r="E28" s="31">
         <f t="shared" si="1"/>
         <v>1938</v>
       </c>
-      <c r="F28" s="32">
+      <c r="F28" s="31">
         <f t="shared" si="2"/>
         <v>0.04817218996</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="25">
+      <c r="A29" s="24">
         <v>1939.0</v>
       </c>
-      <c r="B29" s="25">
+      <c r="B29" s="24">
         <v>13.9</v>
       </c>
-      <c r="C29" s="33">
+      <c r="C29" s="32">
         <v>-0.013</v>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="31">
         <f t="shared" si="1"/>
         <v>1939</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="31">
         <f t="shared" si="2"/>
         <v>0.04748889648</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="25">
+      <c r="A30" s="24">
         <v>1940.0</v>
       </c>
-      <c r="B30" s="25">
+      <c r="B30" s="24">
         <v>14.0</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="32">
         <v>0.007</v>
       </c>
-      <c r="E30" s="32">
+      <c r="E30" s="31">
         <f t="shared" si="1"/>
         <v>1940</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="31">
         <f t="shared" si="2"/>
         <v>0.04783054322</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25">
+      <c r="A31" s="24">
         <v>1941.0</v>
       </c>
-      <c r="B31" s="25">
+      <c r="B31" s="24">
         <v>14.7</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="32">
         <v>0.051</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="31">
         <f t="shared" si="1"/>
         <v>1941</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="31">
         <f t="shared" si="2"/>
         <v>0.05022207038</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="25">
+      <c r="A32" s="24">
         <v>1942.0</v>
       </c>
-      <c r="B32" s="25">
+      <c r="B32" s="24">
         <v>16.3</v>
       </c>
-      <c r="C32" s="33">
+      <c r="C32" s="32">
         <v>0.109</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="31">
         <f t="shared" si="1"/>
         <v>1942</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="31">
         <f t="shared" si="2"/>
         <v>0.05568841818</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="25">
+      <c r="A33" s="24">
         <v>1943.0</v>
       </c>
-      <c r="B33" s="25">
+      <c r="B33" s="24">
         <v>17.3</v>
       </c>
-      <c r="C33" s="33">
+      <c r="C33" s="32">
         <v>0.06</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="31">
         <f t="shared" si="1"/>
         <v>1943</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="31">
         <f t="shared" si="2"/>
         <v>0.05910488555</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="25">
+      <c r="A34" s="24">
         <v>1944.0</v>
       </c>
-      <c r="B34" s="25">
+      <c r="B34" s="24">
         <v>17.6</v>
       </c>
-      <c r="C34" s="33">
+      <c r="C34" s="32">
         <v>0.016</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="31">
         <f t="shared" si="1"/>
         <v>1944</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="31">
         <f t="shared" si="2"/>
         <v>0.06012982576</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="25">
+      <c r="A35" s="24">
         <v>1945.0</v>
       </c>
-      <c r="B35" s="25">
+      <c r="B35" s="24">
         <v>18.0</v>
       </c>
-      <c r="C35" s="33">
+      <c r="C35" s="32">
         <v>0.023</v>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="31">
         <f t="shared" si="1"/>
         <v>1945</v>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="31">
         <f t="shared" si="2"/>
         <v>0.06149641271</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="25">
+      <c r="A36" s="24">
         <v>1946.0</v>
       </c>
-      <c r="B36" s="25">
+      <c r="B36" s="24">
         <v>19.5</v>
       </c>
-      <c r="C36" s="33">
+      <c r="C36" s="32">
         <v>0.085</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="31">
         <f t="shared" si="1"/>
         <v>1946</v>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="31">
         <f t="shared" si="2"/>
         <v>0.06662111377</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="25">
+      <c r="A37" s="24">
         <v>1947.0</v>
       </c>
-      <c r="B37" s="25">
+      <c r="B37" s="24">
         <v>22.3</v>
       </c>
-      <c r="C37" s="33">
+      <c r="C37" s="32">
         <v>0.144</v>
       </c>
-      <c r="E37" s="32">
+      <c r="E37" s="31">
         <f t="shared" si="1"/>
         <v>1947</v>
       </c>
-      <c r="F37" s="32">
+      <c r="F37" s="31">
         <f t="shared" si="2"/>
         <v>0.07618722241</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="25">
+      <c r="A38" s="24">
         <v>1948.0</v>
       </c>
-      <c r="B38" s="25">
+      <c r="B38" s="24">
         <v>24.0</v>
       </c>
-      <c r="C38" s="33">
+      <c r="C38" s="32">
         <v>0.077</v>
       </c>
-      <c r="E38" s="32">
+      <c r="E38" s="31">
         <f t="shared" si="1"/>
         <v>1948</v>
       </c>
-      <c r="F38" s="32">
+      <c r="F38" s="31">
         <f t="shared" si="2"/>
         <v>0.08199521695</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="25">
+      <c r="A39" s="24">
         <v>1949.0</v>
       </c>
-      <c r="B39" s="25">
+      <c r="B39" s="24">
         <v>23.8</v>
       </c>
-      <c r="C39" s="33">
+      <c r="C39" s="32">
         <v>-0.01</v>
       </c>
-      <c r="E39" s="32">
+      <c r="E39" s="31">
         <f t="shared" si="1"/>
         <v>1949</v>
       </c>
-      <c r="F39" s="32">
+      <c r="F39" s="31">
         <f t="shared" si="2"/>
         <v>0.08131192347</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="25">
+      <c r="A40" s="24">
         <v>1950.0</v>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="24">
         <v>24.1</v>
       </c>
-      <c r="C40" s="33">
+      <c r="C40" s="32">
         <v>0.011</v>
       </c>
-      <c r="E40" s="32">
+      <c r="E40" s="31">
         <f t="shared" si="1"/>
         <v>1950</v>
       </c>
-      <c r="F40" s="32">
+      <c r="F40" s="31">
         <f t="shared" si="2"/>
         <v>0.08233686368</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="25">
+      <c r="A41" s="24">
         <v>1951.0</v>
       </c>
-      <c r="B41" s="25">
+      <c r="B41" s="24">
         <v>26.0</v>
       </c>
-      <c r="C41" s="33">
+      <c r="C41" s="32">
         <v>0.079</v>
       </c>
-      <c r="E41" s="32">
+      <c r="E41" s="31">
         <f t="shared" si="1"/>
         <v>1951</v>
       </c>
-      <c r="F41" s="32">
+      <c r="F41" s="31">
         <f t="shared" si="2"/>
         <v>0.08882815169</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="25">
+      <c r="A42" s="24">
         <v>1952.0</v>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="24">
         <v>26.6</v>
       </c>
-      <c r="C42" s="33">
+      <c r="C42" s="32">
         <v>0.023</v>
       </c>
-      <c r="E42" s="32">
+      <c r="E42" s="31">
         <f t="shared" si="1"/>
         <v>1952</v>
       </c>
-      <c r="F42" s="32">
+      <c r="F42" s="31">
         <f t="shared" si="2"/>
         <v>0.09087803211</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25">
+      <c r="A43" s="24">
         <v>1953.0</v>
       </c>
-      <c r="B43" s="25">
+      <c r="B43" s="24">
         <v>26.8</v>
       </c>
-      <c r="C43" s="33">
+      <c r="C43" s="32">
         <v>0.008</v>
       </c>
-      <c r="E43" s="32">
+      <c r="E43" s="31">
         <f t="shared" si="1"/>
         <v>1953</v>
       </c>
-      <c r="F43" s="32">
+      <c r="F43" s="31">
         <f t="shared" si="2"/>
         <v>0.09156132559</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="25">
+      <c r="A44" s="24">
         <v>1954.0</v>
       </c>
-      <c r="B44" s="25">
+      <c r="B44" s="24">
         <v>26.9</v>
       </c>
-      <c r="C44" s="33">
+      <c r="C44" s="32">
         <v>0.003</v>
       </c>
-      <c r="E44" s="32">
+      <c r="E44" s="31">
         <f t="shared" si="1"/>
         <v>1954</v>
       </c>
-      <c r="F44" s="32">
+      <c r="F44" s="31">
         <f t="shared" si="2"/>
         <v>0.09190297233</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="25">
+      <c r="A45" s="24">
         <v>1955.0</v>
       </c>
-      <c r="B45" s="25">
+      <c r="B45" s="24">
         <v>26.8</v>
       </c>
-      <c r="C45" s="33">
+      <c r="C45" s="32">
         <v>-0.003</v>
       </c>
-      <c r="E45" s="32">
+      <c r="E45" s="31">
         <f t="shared" si="1"/>
         <v>1955</v>
       </c>
-      <c r="F45" s="32">
+      <c r="F45" s="31">
         <f t="shared" si="2"/>
         <v>0.09156132559</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="25">
+      <c r="A46" s="24">
         <v>1956.0</v>
       </c>
-      <c r="B46" s="25">
+      <c r="B46" s="24">
         <v>27.2</v>
       </c>
-      <c r="C46" s="33">
+      <c r="C46" s="32">
         <v>0.015</v>
       </c>
-      <c r="E46" s="32">
+      <c r="E46" s="31">
         <f t="shared" si="1"/>
         <v>1956</v>
       </c>
-      <c r="F46" s="32">
+      <c r="F46" s="31">
         <f t="shared" si="2"/>
         <v>0.09292791254</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25">
+      <c r="A47" s="24">
         <v>1957.0</v>
       </c>
-      <c r="B47" s="25">
+      <c r="B47" s="24">
         <v>28.1</v>
       </c>
-      <c r="C47" s="33">
+      <c r="C47" s="32">
         <v>0.033</v>
       </c>
-      <c r="E47" s="32">
+      <c r="E47" s="31">
         <f t="shared" si="1"/>
         <v>1957</v>
       </c>
-      <c r="F47" s="32">
+      <c r="F47" s="31">
         <f t="shared" si="2"/>
         <v>0.09600273317</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25">
+      <c r="A48" s="24">
         <v>1958.0</v>
       </c>
-      <c r="B48" s="25">
+      <c r="B48" s="24">
         <v>28.9</v>
       </c>
-      <c r="C48" s="33">
+      <c r="C48" s="32">
         <v>0.027</v>
       </c>
-      <c r="E48" s="32">
+      <c r="E48" s="31">
         <f t="shared" si="1"/>
         <v>1958</v>
       </c>
-      <c r="F48" s="32">
+      <c r="F48" s="31">
         <f t="shared" si="2"/>
         <v>0.09873590707</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="25">
+      <c r="A49" s="24">
         <v>1959.0</v>
       </c>
-      <c r="B49" s="25">
+      <c r="B49" s="24">
         <v>29.2</v>
       </c>
-      <c r="C49" s="33">
+      <c r="C49" s="32">
         <v>0.0108</v>
       </c>
-      <c r="E49" s="32">
+      <c r="E49" s="31">
         <f t="shared" si="1"/>
         <v>1959</v>
       </c>
-      <c r="F49" s="32">
+      <c r="F49" s="31">
         <f t="shared" si="2"/>
         <v>0.09976084728</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="25">
+      <c r="A50" s="24">
         <v>1960.0</v>
       </c>
-      <c r="B50" s="25">
+      <c r="B50" s="24">
         <v>29.6</v>
       </c>
-      <c r="C50" s="33">
+      <c r="C50" s="32">
         <v>0.015</v>
       </c>
-      <c r="E50" s="32">
+      <c r="E50" s="31">
         <f t="shared" si="1"/>
         <v>1960</v>
       </c>
-      <c r="F50" s="32">
+      <c r="F50" s="31">
         <f t="shared" si="2"/>
         <v>0.1011274342</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="25">
+      <c r="A51" s="24">
         <v>1961.0</v>
       </c>
-      <c r="B51" s="25">
+      <c r="B51" s="24">
         <v>29.9</v>
       </c>
-      <c r="C51" s="33">
+      <c r="C51" s="32">
         <v>0.011</v>
       </c>
-      <c r="E51" s="32">
+      <c r="E51" s="31">
         <f t="shared" si="1"/>
         <v>1961</v>
       </c>
-      <c r="F51" s="32">
+      <c r="F51" s="31">
         <f t="shared" si="2"/>
         <v>0.1021523744</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25">
+      <c r="A52" s="24">
         <v>1962.0</v>
       </c>
-      <c r="B52" s="25">
+      <c r="B52" s="24">
         <v>30.3</v>
       </c>
-      <c r="C52" s="33">
+      <c r="C52" s="32">
         <v>0.012</v>
       </c>
-      <c r="E52" s="32">
+      <c r="E52" s="31">
         <f t="shared" si="1"/>
         <v>1962</v>
       </c>
-      <c r="F52" s="32">
+      <c r="F52" s="31">
         <f t="shared" si="2"/>
         <v>0.1035189614</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="25">
+      <c r="A53" s="24">
         <v>1963.0</v>
       </c>
-      <c r="B53" s="25">
+      <c r="B53" s="24">
         <v>30.6</v>
       </c>
-      <c r="C53" s="33">
+      <c r="C53" s="32">
         <v>0.012</v>
       </c>
-      <c r="E53" s="32">
+      <c r="E53" s="31">
         <f t="shared" si="1"/>
         <v>1963</v>
       </c>
-      <c r="F53" s="32">
+      <c r="F53" s="31">
         <f t="shared" si="2"/>
         <v>0.1045439016</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="25">
+      <c r="A54" s="24">
         <v>1964.0</v>
       </c>
-      <c r="B54" s="25">
+      <c r="B54" s="24">
         <v>31.0</v>
       </c>
-      <c r="C54" s="33">
+      <c r="C54" s="32">
         <v>0.013</v>
       </c>
-      <c r="E54" s="32">
+      <c r="E54" s="31">
         <f t="shared" si="1"/>
         <v>1964</v>
       </c>
-      <c r="F54" s="32">
+      <c r="F54" s="31">
         <f t="shared" si="2"/>
         <v>0.1059104886</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="25">
+      <c r="A55" s="24">
         <v>1965.0</v>
       </c>
-      <c r="B55" s="25">
+      <c r="B55" s="24">
         <v>31.5</v>
       </c>
-      <c r="C55" s="33">
+      <c r="C55" s="32">
         <v>0.016</v>
       </c>
-      <c r="E55" s="32">
+      <c r="E55" s="31">
         <f t="shared" si="1"/>
         <v>1965</v>
       </c>
-      <c r="F55" s="32">
+      <c r="F55" s="31">
         <f t="shared" si="2"/>
         <v>0.1076187222</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="25">
+      <c r="A56" s="24">
         <v>1966.0</v>
       </c>
-      <c r="B56" s="25">
+      <c r="B56" s="24">
         <v>32.5</v>
       </c>
-      <c r="C56" s="33">
+      <c r="C56" s="32">
         <v>0.03</v>
       </c>
-      <c r="E56" s="32">
+      <c r="E56" s="31">
         <f t="shared" si="1"/>
         <v>1966</v>
       </c>
-      <c r="F56" s="32">
+      <c r="F56" s="31">
         <f t="shared" si="2"/>
         <v>0.1110351896</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="25">
+      <c r="A57" s="24">
         <v>1967.0</v>
       </c>
-      <c r="B57" s="25">
+      <c r="B57" s="24">
         <v>33.4</v>
       </c>
-      <c r="C57" s="33">
+      <c r="C57" s="32">
         <v>0.028</v>
       </c>
-      <c r="E57" s="32">
+      <c r="E57" s="31">
         <f t="shared" si="1"/>
         <v>1967</v>
       </c>
-      <c r="F57" s="32">
+      <c r="F57" s="31">
         <f t="shared" si="2"/>
         <v>0.1141100102</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="25">
+      <c r="A58" s="24">
         <v>1968.0</v>
       </c>
-      <c r="B58" s="25">
+      <c r="B58" s="24">
         <v>34.8</v>
       </c>
-      <c r="C58" s="33">
+      <c r="C58" s="32">
         <v>0.043</v>
       </c>
-      <c r="E58" s="32">
+      <c r="E58" s="31">
         <f t="shared" si="1"/>
         <v>1968</v>
       </c>
-      <c r="F58" s="32">
+      <c r="F58" s="31">
         <f t="shared" si="2"/>
         <v>0.1188930646</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25">
+      <c r="A59" s="24">
         <v>1969.0</v>
       </c>
-      <c r="B59" s="25">
+      <c r="B59" s="24">
         <v>36.7</v>
       </c>
-      <c r="C59" s="33">
+      <c r="C59" s="32">
         <v>0.055</v>
       </c>
-      <c r="E59" s="32">
+      <c r="E59" s="31">
         <f t="shared" si="1"/>
         <v>1969</v>
       </c>
-      <c r="F59" s="32">
+      <c r="F59" s="31">
         <f t="shared" si="2"/>
         <v>0.1253843526</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="25">
+      <c r="A60" s="24">
         <v>1970.0</v>
       </c>
-      <c r="B60" s="25">
+      <c r="B60" s="24">
         <v>38.8</v>
       </c>
-      <c r="C60" s="33">
+      <c r="C60" s="32">
         <v>0.058</v>
       </c>
-      <c r="E60" s="32">
+      <c r="E60" s="31">
         <f t="shared" si="1"/>
         <v>1970</v>
       </c>
-      <c r="F60" s="32">
+      <c r="F60" s="31">
         <f t="shared" si="2"/>
         <v>0.1325589341</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="25">
+      <c r="A61" s="24">
         <v>1971.0</v>
       </c>
-      <c r="B61" s="25">
+      <c r="B61" s="24">
         <v>40.5</v>
       </c>
-      <c r="C61" s="33">
+      <c r="C61" s="32">
         <v>0.043</v>
       </c>
-      <c r="E61" s="32">
+      <c r="E61" s="31">
         <f t="shared" si="1"/>
         <v>1971</v>
       </c>
-      <c r="F61" s="32">
+      <c r="F61" s="31">
         <f t="shared" si="2"/>
         <v>0.1383669286</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="25">
+      <c r="A62" s="24">
         <v>1972.0</v>
       </c>
-      <c r="B62" s="25">
+      <c r="B62" s="24">
         <v>41.8</v>
       </c>
-      <c r="C62" s="33">
+      <c r="C62" s="32">
         <v>0.033</v>
       </c>
-      <c r="E62" s="32">
+      <c r="E62" s="31">
         <f t="shared" si="1"/>
         <v>1972</v>
       </c>
-      <c r="F62" s="32">
+      <c r="F62" s="31">
         <f t="shared" si="2"/>
         <v>0.1428083362</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="25">
+      <c r="A63" s="24">
         <v>1973.0</v>
       </c>
-      <c r="B63" s="25">
+      <c r="B63" s="24">
         <v>44.4</v>
       </c>
-      <c r="C63" s="33">
+      <c r="C63" s="32">
         <v>0.062</v>
       </c>
-      <c r="E63" s="32">
+      <c r="E63" s="31">
         <f t="shared" si="1"/>
         <v>1973</v>
       </c>
-      <c r="F63" s="32">
+      <c r="F63" s="31">
         <f t="shared" si="2"/>
         <v>0.1516911513</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="25">
+      <c r="A64" s="24">
         <v>1974.0</v>
       </c>
-      <c r="B64" s="25">
+      <c r="B64" s="24">
         <v>49.3</v>
       </c>
-      <c r="C64" s="33">
+      <c r="C64" s="32">
         <v>0.111</v>
       </c>
-      <c r="E64" s="32">
+      <c r="E64" s="31">
         <f t="shared" si="1"/>
         <v>1974</v>
       </c>
-      <c r="F64" s="32">
+      <c r="F64" s="31">
         <f t="shared" si="2"/>
         <v>0.1684318415</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="25">
+      <c r="A65" s="24">
         <v>1975.0</v>
       </c>
-      <c r="B65" s="25">
+      <c r="B65" s="24">
         <v>53.8</v>
       </c>
-      <c r="C65" s="33">
+      <c r="C65" s="32">
         <v>0.091</v>
       </c>
-      <c r="E65" s="32">
+      <c r="E65" s="31">
         <f t="shared" si="1"/>
         <v>1975</v>
       </c>
-      <c r="F65" s="32">
+      <c r="F65" s="31">
         <f t="shared" si="2"/>
         <v>0.1838059447</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="25">
+      <c r="A66" s="24">
         <v>1976.0</v>
       </c>
-      <c r="B66" s="25">
+      <c r="B66" s="24">
         <v>56.9</v>
       </c>
-      <c r="C66" s="33">
+      <c r="C66" s="32">
         <v>0.057</v>
       </c>
-      <c r="E66" s="32">
+      <c r="E66" s="31">
         <f t="shared" si="1"/>
         <v>1976</v>
       </c>
-      <c r="F66" s="32">
+      <c r="F66" s="31">
         <f t="shared" si="2"/>
         <v>0.1943969935</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="25">
+      <c r="A67" s="24">
         <v>1977.0</v>
       </c>
-      <c r="B67" s="25">
+      <c r="B67" s="24">
         <v>60.6</v>
       </c>
-      <c r="C67" s="33">
+      <c r="C67" s="32">
         <v>0.065</v>
       </c>
-      <c r="E67" s="32">
+      <c r="E67" s="31">
         <f t="shared" si="1"/>
         <v>1977</v>
       </c>
-      <c r="F67" s="32">
+      <c r="F67" s="31">
         <f t="shared" si="2"/>
         <v>0.2070379228</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="25">
+      <c r="A68" s="24">
         <v>1978.0</v>
       </c>
-      <c r="B68" s="25">
+      <c r="B68" s="24">
         <v>65.2</v>
       </c>
-      <c r="C68" s="33">
+      <c r="C68" s="32">
         <v>0.076</v>
       </c>
-      <c r="E68" s="32">
+      <c r="E68" s="31">
         <f t="shared" si="1"/>
         <v>1978</v>
       </c>
-      <c r="F68" s="32">
+      <c r="F68" s="31">
         <f t="shared" si="2"/>
         <v>0.2227536727</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="25">
+      <c r="A69" s="24">
         <v>1979.0</v>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="24">
         <v>72.6</v>
       </c>
-      <c r="C69" s="33">
+      <c r="C69" s="32">
         <v>0.113</v>
       </c>
-      <c r="E69" s="32">
+      <c r="E69" s="31">
         <f t="shared" si="1"/>
         <v>1979</v>
       </c>
-      <c r="F69" s="32">
+      <c r="F69" s="31">
         <f t="shared" si="2"/>
         <v>0.2480355313</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="25">
+      <c r="A70" s="24">
         <v>1980.0</v>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="24">
         <v>82.4</v>
       </c>
-      <c r="C70" s="33">
+      <c r="C70" s="32">
         <v>0.135</v>
       </c>
-      <c r="E70" s="32">
+      <c r="E70" s="31">
         <f t="shared" si="1"/>
         <v>1980</v>
       </c>
-      <c r="F70" s="32">
+      <c r="F70" s="31">
         <f t="shared" si="2"/>
         <v>0.2815169115</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="25">
+      <c r="A71" s="24">
         <v>1981.0</v>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="24">
         <v>90.9</v>
       </c>
-      <c r="C71" s="33">
+      <c r="C71" s="32">
         <v>0.103</v>
       </c>
-      <c r="E71" s="32">
+      <c r="E71" s="31">
         <f t="shared" si="1"/>
         <v>1981</v>
       </c>
-      <c r="F71" s="32">
+      <c r="F71" s="31">
         <f t="shared" si="2"/>
         <v>0.3105568842</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="25">
+      <c r="A72" s="24">
         <v>1982.0</v>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="24">
         <v>96.5</v>
       </c>
-      <c r="C72" s="33">
+      <c r="C72" s="32">
         <v>0.061</v>
       </c>
-      <c r="E72" s="32">
+      <c r="E72" s="31">
         <f t="shared" si="1"/>
         <v>1982</v>
       </c>
-      <c r="F72" s="32">
+      <c r="F72" s="31">
         <f t="shared" si="2"/>
         <v>0.3296891015</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="25">
+      <c r="A73" s="24">
         <v>1983.0</v>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="24">
         <v>99.6</v>
       </c>
-      <c r="C73" s="33">
+      <c r="C73" s="32">
         <v>0.032</v>
       </c>
-      <c r="E73" s="32">
+      <c r="E73" s="31">
         <f t="shared" si="1"/>
         <v>1983</v>
       </c>
-      <c r="F73" s="32">
+      <c r="F73" s="31">
         <f t="shared" si="2"/>
         <v>0.3402801503</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="25">
+      <c r="A74" s="24">
         <v>1984.0</v>
       </c>
-      <c r="B74" s="25">
+      <c r="B74" s="24">
         <v>103.9</v>
       </c>
-      <c r="C74" s="33">
+      <c r="C74" s="32">
         <v>0.043</v>
       </c>
-      <c r="E74" s="32">
+      <c r="E74" s="31">
         <f t="shared" si="1"/>
         <v>1984</v>
       </c>
-      <c r="F74" s="32">
+      <c r="F74" s="31">
         <f t="shared" si="2"/>
         <v>0.35497096</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="25">
+      <c r="A75" s="24">
         <v>1985.0</v>
       </c>
-      <c r="B75" s="25">
+      <c r="B75" s="24">
         <v>107.6</v>
       </c>
-      <c r="C75" s="33">
+      <c r="C75" s="32">
         <v>0.035</v>
       </c>
-      <c r="E75" s="32">
+      <c r="E75" s="31">
         <f t="shared" si="1"/>
         <v>1985</v>
       </c>
-      <c r="F75" s="32">
+      <c r="F75" s="31">
         <f t="shared" si="2"/>
         <v>0.3676118893</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="25">
+      <c r="A76" s="24">
         <v>1986.0</v>
       </c>
-      <c r="B76" s="25">
+      <c r="B76" s="24">
         <v>109.6</v>
       </c>
-      <c r="C76" s="33">
+      <c r="C76" s="32">
         <v>0.019</v>
       </c>
-      <c r="E76" s="32">
+      <c r="E76" s="31">
         <f t="shared" si="1"/>
         <v>1986</v>
       </c>
-      <c r="F76" s="32">
+      <c r="F76" s="31">
         <f t="shared" si="2"/>
         <v>0.3744448241</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="25">
+      <c r="A77" s="24">
         <v>1987.0</v>
       </c>
-      <c r="B77" s="25">
+      <c r="B77" s="24">
         <v>113.6</v>
       </c>
-      <c r="C77" s="33">
+      <c r="C77" s="32">
         <v>0.037</v>
       </c>
-      <c r="E77" s="32">
+      <c r="E77" s="31">
         <f t="shared" si="1"/>
         <v>1987</v>
       </c>
-      <c r="F77" s="32">
+      <c r="F77" s="31">
         <f t="shared" si="2"/>
         <v>0.3881106935</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="25">
+      <c r="A78" s="24">
         <v>1988.0</v>
       </c>
-      <c r="B78" s="25">
+      <c r="B78" s="24">
         <v>118.3</v>
       </c>
-      <c r="C78" s="33">
+      <c r="C78" s="32">
         <v>0.041</v>
       </c>
-      <c r="E78" s="32">
+      <c r="E78" s="31">
         <f t="shared" si="1"/>
         <v>1988</v>
       </c>
-      <c r="F78" s="32">
+      <c r="F78" s="31">
         <f t="shared" si="2"/>
         <v>0.4041680902</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="25">
+      <c r="A79" s="24">
         <v>1989.0</v>
       </c>
-      <c r="B79" s="25">
+      <c r="B79" s="24">
         <v>124.0</v>
       </c>
-      <c r="C79" s="33">
+      <c r="C79" s="32">
         <v>0.048</v>
       </c>
-      <c r="E79" s="32">
+      <c r="E79" s="31">
         <f t="shared" si="1"/>
         <v>1989</v>
       </c>
-      <c r="F79" s="32">
+      <c r="F79" s="31">
         <f t="shared" si="2"/>
         <v>0.4236419542</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="25">
+      <c r="A80" s="24">
         <v>1990.0</v>
       </c>
-      <c r="B80" s="25">
+      <c r="B80" s="24">
         <v>130.7</v>
       </c>
-      <c r="C80" s="33">
+      <c r="C80" s="32">
         <v>0.054</v>
       </c>
-      <c r="E80" s="32">
+      <c r="E80" s="31">
         <f t="shared" si="1"/>
         <v>1990</v>
       </c>
-      <c r="F80" s="32">
+      <c r="F80" s="31">
         <f t="shared" si="2"/>
         <v>0.4465322856</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="25">
+      <c r="A81" s="24">
         <v>1991.0</v>
       </c>
-      <c r="B81" s="25">
+      <c r="B81" s="24">
         <v>136.2</v>
       </c>
-      <c r="C81" s="33">
+      <c r="C81" s="32">
         <v>0.042</v>
       </c>
-      <c r="E81" s="32">
+      <c r="E81" s="31">
         <f t="shared" si="1"/>
         <v>1991</v>
       </c>
-      <c r="F81" s="32">
+      <c r="F81" s="31">
         <f t="shared" si="2"/>
         <v>0.4653228562</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="25">
+      <c r="A82" s="24">
         <v>1992.0</v>
       </c>
-      <c r="B82" s="25">
+      <c r="B82" s="24">
         <v>140.3</v>
       </c>
-      <c r="C82" s="33">
+      <c r="C82" s="32">
         <v>0.03</v>
       </c>
-      <c r="E82" s="32">
+      <c r="E82" s="31">
         <f t="shared" si="1"/>
         <v>1992</v>
       </c>
-      <c r="F82" s="32">
+      <c r="F82" s="31">
         <f t="shared" si="2"/>
         <v>0.4793303724</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="25">
+      <c r="A83" s="24">
         <v>1993.0</v>
       </c>
-      <c r="B83" s="25">
+      <c r="B83" s="24">
         <v>144.5</v>
       </c>
-      <c r="C83" s="33">
+      <c r="C83" s="32">
         <v>0.03</v>
       </c>
-      <c r="E83" s="32">
+      <c r="E83" s="31">
         <f t="shared" si="1"/>
         <v>1993</v>
       </c>
-      <c r="F83" s="32">
+      <c r="F83" s="31">
         <f t="shared" si="2"/>
         <v>0.4936795354</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="25">
+      <c r="A84" s="24">
         <v>1994.0</v>
       </c>
-      <c r="B84" s="25">
+      <c r="B84" s="24">
         <v>148.2</v>
       </c>
-      <c r="C84" s="33">
+      <c r="C84" s="32">
         <v>0.026</v>
       </c>
-      <c r="E84" s="32">
+      <c r="E84" s="31">
         <f t="shared" si="1"/>
         <v>1994</v>
       </c>
-      <c r="F84" s="32">
+      <c r="F84" s="31">
         <f t="shared" si="2"/>
         <v>0.5063204646</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="25">
+      <c r="A85" s="24">
         <v>1995.0</v>
       </c>
-      <c r="B85" s="25">
+      <c r="B85" s="24">
         <v>152.4</v>
       </c>
-      <c r="C85" s="33">
+      <c r="C85" s="32">
         <v>0.028</v>
       </c>
-      <c r="E85" s="32">
+      <c r="E85" s="31">
         <f t="shared" si="1"/>
         <v>1995</v>
       </c>
-      <c r="F85" s="32">
+      <c r="F85" s="31">
         <f t="shared" si="2"/>
         <v>0.5206696276</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="25">
+      <c r="A86" s="24">
         <v>1996.0</v>
       </c>
-      <c r="B86" s="25">
+      <c r="B86" s="24">
         <v>156.9</v>
       </c>
-      <c r="C86" s="33">
+      <c r="C86" s="32">
         <v>0.029</v>
       </c>
-      <c r="E86" s="32">
+      <c r="E86" s="31">
         <f t="shared" si="1"/>
         <v>1996</v>
       </c>
-      <c r="F86" s="32">
+      <c r="F86" s="31">
         <f t="shared" si="2"/>
         <v>0.5360437308</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="25">
+      <c r="A87" s="24">
         <v>1997.0</v>
       </c>
-      <c r="B87" s="25">
+      <c r="B87" s="24">
         <v>160.5</v>
       </c>
-      <c r="C87" s="33">
+      <c r="C87" s="32">
         <v>0.023</v>
       </c>
-      <c r="E87" s="32">
+      <c r="E87" s="31">
         <f t="shared" si="1"/>
         <v>1997</v>
       </c>
-      <c r="F87" s="32">
+      <c r="F87" s="31">
         <f t="shared" si="2"/>
         <v>0.5483430133</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="25">
+      <c r="A88" s="24">
         <v>1998.0</v>
       </c>
-      <c r="B88" s="25">
+      <c r="B88" s="24">
         <v>163.0</v>
       </c>
-      <c r="C88" s="33">
+      <c r="C88" s="32">
         <v>0.016</v>
       </c>
-      <c r="E88" s="32">
+      <c r="E88" s="31">
         <f t="shared" si="1"/>
         <v>1998</v>
       </c>
-      <c r="F88" s="32">
+      <c r="F88" s="31">
         <f t="shared" si="2"/>
         <v>0.5568841818</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="25">
+      <c r="A89" s="24">
         <v>1999.0</v>
       </c>
-      <c r="B89" s="25">
+      <c r="B89" s="24">
         <v>166.6</v>
       </c>
-      <c r="C89" s="33">
+      <c r="C89" s="32">
         <v>0.022</v>
       </c>
-      <c r="E89" s="32">
+      <c r="E89" s="31">
         <f t="shared" si="1"/>
         <v>1999</v>
       </c>
-      <c r="F89" s="32">
+      <c r="F89" s="31">
         <f t="shared" si="2"/>
         <v>0.5691834643</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="25">
+      <c r="A90" s="24">
         <v>2000.0</v>
       </c>
-      <c r="B90" s="25">
+      <c r="B90" s="24">
         <v>172.2</v>
       </c>
-      <c r="C90" s="33">
+      <c r="C90" s="32">
         <v>0.034</v>
       </c>
-      <c r="E90" s="32">
+      <c r="E90" s="31">
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="F90" s="32">
+      <c r="F90" s="31">
         <f t="shared" si="2"/>
         <v>0.5883156816</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="25">
+      <c r="A91" s="24">
         <v>2001.0</v>
       </c>
-      <c r="B91" s="25">
+      <c r="B91" s="24">
         <v>177.1</v>
       </c>
-      <c r="C91" s="33">
+      <c r="C91" s="32">
         <v>0.028</v>
       </c>
-      <c r="E91" s="32">
+      <c r="E91" s="31">
         <f t="shared" si="1"/>
         <v>2001</v>
       </c>
-      <c r="F91" s="32">
+      <c r="F91" s="31">
         <f t="shared" si="2"/>
         <v>0.6050563717</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="25">
+      <c r="A92" s="24">
         <v>2002.0</v>
       </c>
-      <c r="B92" s="25">
+      <c r="B92" s="24">
         <v>179.9</v>
       </c>
-      <c r="C92" s="33">
+      <c r="C92" s="32">
         <v>0.016</v>
       </c>
-      <c r="E92" s="32">
+      <c r="E92" s="31">
         <f t="shared" si="1"/>
         <v>2002</v>
       </c>
-      <c r="F92" s="32">
+      <c r="F92" s="31">
         <f t="shared" si="2"/>
         <v>0.6146224804</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="25">
+      <c r="A93" s="24">
         <v>2003.0</v>
       </c>
-      <c r="B93" s="25">
+      <c r="B93" s="24">
         <v>184.0</v>
       </c>
-      <c r="C93" s="33">
+      <c r="C93" s="32">
         <v>0.023</v>
       </c>
-      <c r="E93" s="32">
+      <c r="E93" s="31">
         <f t="shared" si="1"/>
         <v>2003</v>
       </c>
-      <c r="F93" s="32">
+      <c r="F93" s="31">
         <f t="shared" si="2"/>
         <v>0.6286299966</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="25">
+      <c r="A94" s="24">
         <v>2004.0</v>
       </c>
-      <c r="B94" s="25">
+      <c r="B94" s="24">
         <v>188.9</v>
       </c>
-      <c r="C94" s="33">
+      <c r="C94" s="32">
         <v>0.027</v>
       </c>
-      <c r="E94" s="32">
+      <c r="E94" s="31">
         <f t="shared" si="1"/>
         <v>2004</v>
       </c>
-      <c r="F94" s="32">
+      <c r="F94" s="31">
         <f t="shared" si="2"/>
         <v>0.6453706867</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="25">
+      <c r="A95" s="24">
         <v>2005.0</v>
       </c>
-      <c r="B95" s="25">
+      <c r="B95" s="24">
         <v>195.3</v>
       </c>
-      <c r="C95" s="33">
+      <c r="C95" s="32">
         <v>0.034</v>
       </c>
-      <c r="E95" s="32">
+      <c r="E95" s="31">
         <f t="shared" si="1"/>
         <v>2005</v>
       </c>
-      <c r="F95" s="32">
+      <c r="F95" s="31">
         <f t="shared" si="2"/>
         <v>0.6672360779</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="25">
+      <c r="A96" s="24">
         <v>2006.0</v>
       </c>
-      <c r="B96" s="25">
+      <c r="B96" s="24">
         <v>201.6</v>
       </c>
-      <c r="C96" s="33">
+      <c r="C96" s="32">
         <v>0.032</v>
       </c>
-      <c r="E96" s="32">
+      <c r="E96" s="31">
         <f t="shared" si="1"/>
         <v>2006</v>
       </c>
-      <c r="F96" s="32">
+      <c r="F96" s="31">
         <f t="shared" si="2"/>
         <v>0.6887598223</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="25">
+      <c r="A97" s="24">
         <v>2007.0</v>
       </c>
-      <c r="B97" s="25">
+      <c r="B97" s="24">
         <v>207.3</v>
       </c>
-      <c r="C97" s="33">
+      <c r="C97" s="32">
         <v>0.029</v>
       </c>
-      <c r="E97" s="32">
+      <c r="E97" s="31">
         <f t="shared" si="1"/>
         <v>2007</v>
       </c>
-      <c r="F97" s="32">
+      <c r="F97" s="31">
         <f t="shared" si="2"/>
         <v>0.7082336864</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="25">
+      <c r="A98" s="24">
         <v>2008.0</v>
       </c>
-      <c r="B98" s="25">
+      <c r="B98" s="24">
         <v>215.3</v>
       </c>
-      <c r="C98" s="33">
+      <c r="C98" s="32">
         <v>0.038</v>
       </c>
-      <c r="E98" s="32">
+      <c r="E98" s="31">
         <f t="shared" si="1"/>
         <v>2008</v>
       </c>
-      <c r="F98" s="32">
+      <c r="F98" s="31">
         <f t="shared" si="2"/>
         <v>0.7355654254</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="25">
+      <c r="A99" s="24">
         <v>2009.0</v>
       </c>
-      <c r="B99" s="25">
+      <c r="B99" s="24">
         <v>214.5</v>
       </c>
-      <c r="C99" s="33">
+      <c r="C99" s="32">
         <v>-0.004</v>
       </c>
-      <c r="E99" s="32">
+      <c r="E99" s="31">
         <f t="shared" si="1"/>
         <v>2009</v>
       </c>
-      <c r="F99" s="32">
+      <c r="F99" s="31">
         <f t="shared" si="2"/>
         <v>0.7328322515</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="25">
+      <c r="A100" s="24">
         <v>2010.0</v>
       </c>
-      <c r="B100" s="25">
+      <c r="B100" s="24">
         <v>218.1</v>
       </c>
-      <c r="C100" s="33">
+      <c r="C100" s="32">
         <v>0.016</v>
       </c>
-      <c r="E100" s="32">
+      <c r="E100" s="31">
         <f t="shared" si="1"/>
         <v>2010</v>
       </c>
-      <c r="F100" s="32">
+      <c r="F100" s="31">
         <f t="shared" si="2"/>
         <v>0.745131534</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="25">
+      <c r="A101" s="24">
         <v>2011.0</v>
       </c>
-      <c r="B101" s="25">
+      <c r="B101" s="24">
         <v>224.9</v>
       </c>
-      <c r="C101" s="33">
+      <c r="C101" s="32">
         <v>0.032</v>
       </c>
-      <c r="E101" s="32">
+      <c r="E101" s="31">
         <f t="shared" si="1"/>
         <v>2011</v>
       </c>
-      <c r="F101" s="32">
+      <c r="F101" s="31">
         <f t="shared" si="2"/>
         <v>0.7683635121</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="25">
+      <c r="A102" s="24">
         <v>2012.0</v>
       </c>
-      <c r="B102" s="25">
+      <c r="B102" s="24">
         <v>229.6</v>
       </c>
-      <c r="C102" s="33">
+      <c r="C102" s="32">
         <v>0.021</v>
       </c>
-      <c r="E102" s="32">
+      <c r="E102" s="31">
         <f t="shared" si="1"/>
         <v>2012</v>
       </c>
-      <c r="F102" s="32">
+      <c r="F102" s="31">
         <f t="shared" si="2"/>
         <v>0.7844209088</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="25">
+      <c r="A103" s="24">
         <v>2013.0</v>
       </c>
-      <c r="B103" s="25">
+      <c r="B103" s="24">
         <v>233.0</v>
       </c>
-      <c r="C103" s="33">
+      <c r="C103" s="32">
         <v>0.015</v>
       </c>
-      <c r="E103" s="32">
+      <c r="E103" s="31">
         <f t="shared" si="1"/>
         <v>2013</v>
       </c>
-      <c r="F103" s="32">
+      <c r="F103" s="31">
         <f t="shared" si="2"/>
         <v>0.7960368978</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="25">
+      <c r="A104" s="24">
         <v>2014.0</v>
       </c>
-      <c r="B104" s="25">
+      <c r="B104" s="24">
         <v>236.7</v>
       </c>
-      <c r="C104" s="33">
+      <c r="C104" s="32">
         <v>0.016</v>
       </c>
-      <c r="E104" s="32">
+      <c r="E104" s="31">
         <f t="shared" si="1"/>
         <v>2014</v>
       </c>
-      <c r="F104" s="32">
+      <c r="F104" s="31">
         <f t="shared" si="2"/>
         <v>0.8086778271</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="25">
+      <c r="A105" s="24">
         <v>2015.0</v>
       </c>
-      <c r="B105" s="25">
+      <c r="B105" s="24">
         <v>237.0</v>
       </c>
-      <c r="C105" s="33">
+      <c r="C105" s="32">
         <v>0.001</v>
       </c>
-      <c r="E105" s="32">
+      <c r="E105" s="31">
         <f t="shared" si="1"/>
         <v>2015</v>
       </c>
-      <c r="F105" s="32">
+      <c r="F105" s="31">
         <f t="shared" si="2"/>
         <v>0.8097027673</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="25">
+      <c r="A106" s="24">
         <v>2016.0</v>
       </c>
-      <c r="B106" s="25">
+      <c r="B106" s="24">
         <v>240.0</v>
       </c>
-      <c r="C106" s="33">
+      <c r="C106" s="32">
         <v>0.013</v>
       </c>
-      <c r="E106" s="32">
+      <c r="E106" s="31">
         <f t="shared" si="1"/>
         <v>2016</v>
       </c>
-      <c r="F106" s="32">
+      <c r="F106" s="31">
         <f t="shared" si="2"/>
         <v>0.8199521695</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="25">
+      <c r="A107" s="24">
         <v>2017.0</v>
       </c>
-      <c r="B107" s="25">
+      <c r="B107" s="24">
         <v>245.1</v>
       </c>
-      <c r="C107" s="33">
+      <c r="C107" s="32">
         <v>0.021</v>
       </c>
-      <c r="E107" s="32">
+      <c r="E107" s="31">
         <f t="shared" si="1"/>
         <v>2017</v>
       </c>
-      <c r="F107" s="32">
+      <c r="F107" s="31">
         <f t="shared" si="2"/>
         <v>0.8373761531</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="25">
+      <c r="A108" s="24">
         <v>2018.0</v>
       </c>
-      <c r="B108" s="25">
+      <c r="B108" s="24">
         <v>251.1</v>
       </c>
-      <c r="C108" s="33">
+      <c r="C108" s="32">
         <v>0.024</v>
       </c>
-      <c r="E108" s="32">
+      <c r="E108" s="31">
         <f t="shared" si="1"/>
         <v>2018</v>
       </c>
-      <c r="F108" s="32">
+      <c r="F108" s="31">
         <f t="shared" si="2"/>
         <v>0.8578749573</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="25">
+      <c r="A109" s="24">
         <v>2019.0</v>
       </c>
-      <c r="B109" s="25">
+      <c r="B109" s="24">
         <v>255.7</v>
       </c>
-      <c r="C109" s="33">
+      <c r="C109" s="32">
         <v>0.018</v>
       </c>
-      <c r="E109" s="32">
+      <c r="E109" s="31">
         <f t="shared" si="1"/>
         <v>2019</v>
       </c>
-      <c r="F109" s="32">
+      <c r="F109" s="31">
         <f t="shared" si="2"/>
         <v>0.8735907072</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="25">
+      <c r="A110" s="24">
         <v>2020.0</v>
       </c>
-      <c r="B110" s="25">
+      <c r="B110" s="24">
         <v>258.8</v>
       </c>
-      <c r="C110" s="33">
+      <c r="C110" s="32">
         <v>0.012</v>
       </c>
-      <c r="E110" s="32">
+      <c r="E110" s="31">
         <f t="shared" si="1"/>
         <v>2020</v>
       </c>
-      <c r="F110" s="32">
+      <c r="F110" s="31">
         <f t="shared" si="2"/>
         <v>0.8841817561</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="25">
+      <c r="A111" s="24">
         <v>2021.0</v>
       </c>
-      <c r="B111" s="25">
+      <c r="B111" s="24">
         <v>271.0</v>
       </c>
-      <c r="C111" s="33">
+      <c r="C111" s="32">
         <v>0.047</v>
       </c>
-      <c r="E111" s="32">
+      <c r="E111" s="31">
         <f t="shared" si="1"/>
         <v>2021</v>
       </c>
-      <c r="F111" s="32">
+      <c r="F111" s="31">
         <f t="shared" si="2"/>
         <v>0.925862658</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="25">
+      <c r="A112" s="24">
         <v>2022.0</v>
       </c>
-      <c r="B112" s="25">
+      <c r="B112" s="24">
         <v>292.7</v>
       </c>
-      <c r="C112" s="33">
+      <c r="C112" s="32">
         <v>0.08</v>
       </c>
-      <c r="E112" s="32">
+      <c r="E112" s="31">
         <f t="shared" si="1"/>
         <v>2022</v>
       </c>
-      <c r="F112" s="32">
+      <c r="F112" s="31">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="25">
+      <c r="A113" s="24">
         <v>2023.0</v>
       </c>
-      <c r="B113" s="25">
+      <c r="B113" s="24">
         <v>304.7</v>
       </c>
-      <c r="C113" s="33">
+      <c r="C113" s="32">
         <v>0.041</v>
       </c>
-      <c r="E113" s="32">
+      <c r="E113" s="31">
         <f t="shared" si="1"/>
         <v>2023</v>
       </c>
-      <c r="F113" s="32">
+      <c r="F113" s="31">
         <f t="shared" si="2"/>
         <v>1.040997608</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="25">
+      <c r="A114" s="24">
         <v>2024.0</v>
       </c>
-      <c r="B114" s="25">
+      <c r="B114" s="24">
         <v>314.4</v>
       </c>
-      <c r="C114" s="33">
+      <c r="C114" s="32">
         <v>0.032</v>
       </c>
-      <c r="E114" s="32">
+      <c r="E114" s="31">
         <f t="shared" si="1"/>
         <v>2024</v>
       </c>
-      <c r="F114" s="32">
+      <c r="F114" s="31">
         <f t="shared" si="2"/>
         <v>1.074137342</v>
       </c>

</xml_diff>

<commit_message>
economic loss model and other changes
</commit_message>
<xml_diff>
--- a/data/raw/Economic damages source review.xlsx
+++ b/data/raw/Economic damages source review.xlsx
@@ -18,10 +18,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={7ccb34cb-dade-4c7f-8ebb-492ad413645c}</author>
+    <author>tc={23e781c9-f373-4e44-b466-a7732ed051cd}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{7ccb34cb-dade-4c7f-8ebb-492ad413645c}" ref="H3">
+    <comment authorId="0" xr:uid="{23e781c9-f373-4e44-b466-a7732ed051cd}" ref="H3">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -37,14 +37,14 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={013c9f1d-f741-4dfd-bca7-0544cb543c28}</author>
-    <author>tc={1d09f527-e964-4af7-8c66-0de839779ce0}</author>
-    <author>tc={1d4bb765-95cc-4c9d-a9b0-62bf4b6eb0e4}</author>
-    <author>tc={36143d33-3642-4511-98d1-6d6ca267d179}</author>
-    <author>tc={f4d0fb94-5c2e-44ac-9b3d-646b49ec2a67}</author>
+    <author>tc={33f4f2c8-bc3d-42e8-b53c-9490dca7db3d}</author>
+    <author>tc={901c1798-7ef0-4e01-9014-63c03c10e409}</author>
+    <author>tc={bddbef71-f3b3-4dd1-b111-2eb11347bbb0}</author>
+    <author>tc={c3881965-75a1-478c-ab4f-5bd714788aac}</author>
+    <author>tc={ef501a19-e989-4c19-8953-2661ee06ee97}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{013c9f1d-f741-4dfd-bca7-0544cb543c28}" ref="H3">
+    <comment authorId="0" xr:uid="{33f4f2c8-bc3d-42e8-b53c-9490dca7db3d}" ref="H3">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -53,7 +53,25 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{1d09f527-e964-4af7-8c66-0de839779ce0}" ref="C8">
+    <comment authorId="1" xr:uid="{901c1798-7ef0-4e01-9014-63c03c10e409}" ref="J8">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Should also interpolate
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{bddbef71-f3b3-4dd1-b111-2eb11347bbb0}" ref="J6">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Should actually interpolate to get this, but approximately right for now
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{c3881965-75a1-478c-ab4f-5bd714788aac}" ref="C8">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,16 +80,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{1d4bb765-95cc-4c9d-a9b0-62bf4b6eb0e4}" ref="J6">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Should actually interpolate to get this, but approximately right for now
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{36143d33-3642-4511-98d1-6d6ca267d179}" ref="K1">
+    <comment authorId="4" xr:uid="{ef501a19-e989-4c19-8953-2661ee06ee97}" ref="K1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -82,21 +91,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="4" xr:uid="{f4d0fb94-5c2e-44ac-9b3d-646b49ec2a67}" ref="J8">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Should also interpolate
-</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="77">
   <si>
     <r>
       <rPr/>
@@ -291,10 +291,13 @@
     <t>Total GDP losses (reference year value, 2024 dollars)</t>
   </si>
   <si>
-    <t>Fraction GDP losses</t>
+    <t>Total GDP over duration (2024 dollars)</t>
   </si>
   <si>
     <t>Annual fraction GPD losses</t>
+  </si>
+  <si>
+    <t>Fraction output loss over total horizon</t>
   </si>
   <si>
     <t>Other notes</t>
@@ -349,7 +352,7 @@
     <t>Marani et al. (Ganqi note)</t>
   </si>
   <si>
-    <t>Sums direct economics costs, treatment and screening costs, and cost of human resources deployment in Huber, Finelli, and Stevens. Multiplies by three to account for three year duration</t>
+    <t>Takes direct economic costs from Huber, Finelli, and Stevens. Multiplies by four to account for three year duration.</t>
   </si>
   <si>
     <r>
@@ -380,7 +383,7 @@
     </r>
   </si>
   <si>
-    <t>Total GDP loss value stated in Agarwal and Gopinath.</t>
+    <t>Total GDP loss value stated in Agarwal and Gopinath. DIvide by sum of GDP over same period.</t>
   </si>
   <si>
     <r>
@@ -389,7 +392,7 @@
         <color rgb="FF000000"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve">Other sources noted by </t>
+      <t xml:space="preserve">4.3% + (4.3% + 1.6%) + (4.3% + 1.6% + 0.5%) total shortfall, divided by three year duration. Other sources noted by </t>
     </r>
     <r>
       <rPr>
@@ -417,6 +420,9 @@
   </si>
   <si>
     <t>Jinjarak et al. (2022)</t>
+  </si>
+  <si>
+    <t>1.2% + (1.2% + 1.2%) cumulative shortfall for 1968-69 period estimated. Then didide by three for 1969-70 duration.</t>
   </si>
   <si>
     <t>Swine flu</t>
@@ -546,12 +552,12 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
-      <name val="&quot;Aptos Narrow&quot;"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
       <b/>
@@ -631,8 +637,9 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="11" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="10" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -660,13 +667,12 @@
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="11" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -765,7 +771,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Updated numbers'!$L$1:$L$9</c:f>
+              <c:f>'Updated numbers'!$N$1:$N$9</c:f>
               <c:numCache/>
             </c:numRef>
           </c:yVal>
@@ -778,11 +784,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1225661372"/>
-        <c:axId val="1717409503"/>
+        <c:axId val="758859341"/>
+        <c:axId val="78381904"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1225661372"/>
+        <c:axId val="758859341"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -857,10 +863,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1717409503"/>
+        <c:crossAx val="78381904"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1717409503"/>
+        <c:axId val="78381904"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.3"/>
@@ -936,7 +942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1225661372"/>
+        <c:crossAx val="758859341"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1022,7 +1028,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Sebastian Barungi Rugunda Quaade" id="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" providerId="google-sheets"/>
+  <x18tc:person displayName="Sebastian Barungi Quaade" id="{1f26886f-dc92-4479-80d5-276f120fe430}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1222,7 +1228,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="H3" dT="2024-10-14T17:20:56.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{7ccb34cb-dade-4c7f-8ebb-492ad413645c}" done="0">
+  <x18tc:threadedComment ref="H3" dT="2024-10-14T17:20:56.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{23e781c9-f373-4e44-b466-a7732ed051cd}" done="0">
     <x18tc:text xml:space="preserve">Should we update to our minimum threshold?</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1230,22 +1236,22 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="J6" dT="2024-10-16T01:28:34.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{1d4bb765-95cc-4c9d-a9b0-62bf4b6eb0e4}" done="0">
+  <x18tc:threadedComment ref="J6" dT="2024-10-16T01:28:34.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{bddbef71-f3b3-4dd1-b111-2eb11347bbb0}" done="0">
     <x18tc:text xml:space="preserve">Should actually interpolate to get this, but approximately right for now</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K1" dT="2024-10-16T01:40:34.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{36143d33-3642-4511-98d1-6d6ca267d179}" done="1">
+  <x18tc:threadedComment ref="K1" dT="2024-10-16T01:40:34.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{ef501a19-e989-4c19-8953-2661ee06ee97}" done="1">
     <x18tc:text xml:space="preserve">We adjust for inflation using urban US CPI</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K1" dT="2024-10-16T03:00:21.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{709fdb68-3c2a-4b23-94b5-4f9730f0cb14}" parentId="{36143d33-3642-4511-98d1-6d6ca267d179}">
+  <x18tc:threadedComment ref="K1" dT="2024-10-16T03:00:21.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{6f6c7785-2d58-4bd3-99f5-990d97f2da5b}" parentId="{ef501a19-e989-4c19-8953-2661ee06ee97}">
     <x18tc:text xml:space="preserve">Also need to adjust for OWID CPI numbers. Do this tomorrow</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="C8" dT="2024-10-16T01:55:59.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{1d09f527-e964-4af7-8c66-0de839779ce0}" done="0">
+  <x18tc:threadedComment ref="C8" dT="2024-10-16T01:55:59.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{c3881965-75a1-478c-ab4f-5bd714788aac}" done="0">
     <x18tc:text xml:space="preserve">Marani et al. data says 1969, but paper for economic losses says 1970</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J8" dT="2024-10-16T01:56:46.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{f4d0fb94-5c2e-44ac-9b3d-646b49ec2a67}" done="0">
+  <x18tc:threadedComment ref="J8" dT="2024-10-16T01:56:46.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{901c1798-7ef0-4e01-9014-63c03c10e409}" done="0">
     <x18tc:text xml:space="preserve">Should also interpolate</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="H3" dT="2024-10-16T01:33:51.00" personId="{78aa5991-85cc-4f85-8852-6f9d2221a9a8}" id="{013c9f1d-f741-4dfd-bca7-0544cb543c28}" done="0">
+  <x18tc:threadedComment ref="H3" dT="2024-10-16T01:33:51.00" personId="{1f26886f-dc92-4479-80d5-276f120fe430}" id="{33f4f2c8-bc3d-42e8-b53c-9490dca7db3d}" done="0">
     <x18tc:text xml:space="preserve">This is a guess since they don't document the reference year for their valuations</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1532,11 +1538,11 @@
     <col customWidth="1" min="7" max="9" width="21.63"/>
     <col customWidth="1" min="10" max="10" width="18.75"/>
     <col customWidth="1" min="11" max="11" width="18.38"/>
-    <col customWidth="1" min="12" max="13" width="16.5"/>
-    <col customWidth="1" min="14" max="14" width="38.5"/>
-    <col customWidth="1" min="15" max="15" width="18.88"/>
-    <col customWidth="1" min="16" max="16" width="33.0"/>
-    <col customWidth="1" min="17" max="17" width="30.13"/>
+    <col customWidth="1" min="12" max="14" width="16.5"/>
+    <col customWidth="1" min="15" max="15" width="38.5"/>
+    <col customWidth="1" min="16" max="16" width="18.88"/>
+    <col customWidth="1" min="17" max="17" width="33.0"/>
+    <col customWidth="1" min="18" max="18" width="30.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1580,18 +1586,20 @@
         <v>39</v>
       </c>
       <c r="N1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="R1" s="4"/>
+      <c r="R1" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="S1" s="4"/>
       <c r="T1" s="4"/>
       <c r="U1" s="4"/>
@@ -1606,6 +1614,7 @@
       <c r="AD1" s="4"/>
       <c r="AE1" s="4"/>
       <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
@@ -1635,33 +1644,37 @@
       <c r="I2" s="6">
         <v>2015.0</v>
       </c>
-      <c r="J2" s="6">
+      <c r="J2" s="15">
         <f>7*1000000000</f>
         <v>7000000000</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="15">
         <f>J2*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I2,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>8645147679</v>
+        <v>9286075949</v>
       </c>
       <c r="L2" s="16">
-        <f>K2/VLOOKUP(H2,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
-        <v>0.0000635021097</v>
+        <f>SUMPRODUCT(  --('Global GDP over time'!C2:C200&gt;=B2),  --('Global GDP over time'!C2:C200&lt;=C2),  'Global GDP over time'!D2:D200 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A3:B114,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A3:B114,2,FALSE))</f>
+        <v>455373317013464</v>
       </c>
       <c r="M2" s="17">
-        <f t="shared" ref="M2:M6" si="3">L2/D2</f>
-        <v>0.0000211673699</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="O2" s="8" t="s">
+        <f t="shared" ref="M2:M6" si="3">N2</f>
+        <v>0.00002039222678</v>
+      </c>
+      <c r="N2" s="18">
+        <f t="shared" ref="N2:N5" si="4">K2/L2</f>
+        <v>0.00002039222678</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="P2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="7" t="s">
         <v>43</v>
+      </c>
+      <c r="R2" s="13" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -1679,7 +1692,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="6"/>
-      <c r="F3" s="18">
+      <c r="F3" s="19">
         <v>0.00116592761933782</v>
       </c>
       <c r="G3" s="6">
@@ -1692,32 +1705,36 @@
       <c r="I3" s="6">
         <v>2005.0</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="15">
         <f>11.8*1000000000</f>
         <v>11800000000</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="15">
         <f>J3*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I3,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>17684895033</v>
+        <v>18996006144</v>
       </c>
       <c r="L3" s="16">
-        <f>K3/VLOOKUP(H3,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
-        <v>0.0001808169642</v>
-      </c>
-      <c r="M3" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C3:C201&gt;=B3),  --('Global GDP over time'!C3:C201&lt;=C3),  'Global GDP over time'!D3:D201 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A4:B115,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A4:B115,2,FALSE))</f>
+        <v>187921664626683</v>
+      </c>
+      <c r="M3" s="17">
         <f t="shared" si="3"/>
-        <v>0.00009040848211</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" s="9" t="s">
+        <v>0.0001010847056</v>
+      </c>
+      <c r="N3" s="18">
+        <f t="shared" si="4"/>
+        <v>0.0001010847056</v>
+      </c>
+      <c r="O3" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="Q3" s="13"/>
+      <c r="Q3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" s="13"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
@@ -1749,32 +1766,36 @@
       <c r="I4" s="6">
         <v>2014.0</v>
       </c>
-      <c r="J4" s="6">
-        <f>15.67*3*1000000000</f>
-        <v>47010000000</v>
-      </c>
-      <c r="K4" s="6">
+      <c r="J4" s="15">
+        <f>14*1000000000</f>
+        <v>14000000000</v>
+      </c>
+      <c r="K4" s="15">
         <f>J4*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I4,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>58131926489</v>
+        <v>18595690748</v>
       </c>
       <c r="L4" s="16">
-        <f>K4/VLOOKUP(H4,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
-        <v>0.0004385431439</v>
-      </c>
-      <c r="M4" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C4:C202&gt;=B4),  --('Global GDP over time'!C4:C202&lt;=C4),  'Global GDP over time'!D4:D202 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A5:B116,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A5:B116,2,FALSE))</f>
+        <v>577233782129743</v>
+      </c>
+      <c r="M4" s="17">
         <f t="shared" si="3"/>
-        <v>0.000109635786</v>
-      </c>
-      <c r="N4" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="O4" s="10" t="s">
+        <v>0.00003221518096</v>
+      </c>
+      <c r="N4" s="18">
+        <f t="shared" si="4"/>
+        <v>0.00003221518096</v>
+      </c>
+      <c r="O4" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="P4" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q4" s="14"/>
+      <c r="Q4" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="R4" s="14"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
@@ -1806,32 +1827,36 @@
       <c r="I5" s="6">
         <v>2019.0</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="15">
         <f>13800000000000</f>
         <v>13800000000000</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="15">
         <f>J5*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I5,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>15796871333594</v>
+        <v>16968009385999</v>
       </c>
       <c r="L5" s="16">
-        <f>K5/VLOOKUP(H5,'Global GDP over time'!$C$1:$E$49,3,FALSE)</f>
-        <v>0.1009765141</v>
-      </c>
-      <c r="M5" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C5:C203&gt;=B5),  --('Global GDP over time'!C5:C203&lt;=C5),  'Global GDP over time'!D5:D203 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A6:B117,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A6:B117,2,FALSE))</f>
+        <v>682418604651163</v>
+      </c>
+      <c r="M5" s="17">
         <f t="shared" si="3"/>
-        <v>0.01682941902</v>
-      </c>
-      <c r="N5" s="10" t="s">
+        <v>0.02486451757</v>
+      </c>
+      <c r="N5" s="18">
+        <f t="shared" si="4"/>
+        <v>0.02486451757</v>
+      </c>
+      <c r="O5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="Q5" s="14"/>
+      <c r="Q5" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="R5" s="14"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
@@ -1862,37 +1887,42 @@
       </c>
       <c r="I6" s="6">
         <f>Constants!$B$1</f>
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="J6" s="15">
-        <f>L6*VLOOKUP(H6, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
-        <v>300223500612</v>
+        <f>N6*VLOOKUP(H6, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
+        <v>297399396165</v>
       </c>
       <c r="K6" s="15">
         <f>J6*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I6,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>300223500612</v>
-      </c>
-      <c r="L6" s="21">
-        <v>0.06</v>
-      </c>
-      <c r="M6" s="16">
+        <v>297399396165</v>
+      </c>
+      <c r="L6" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C6:C204&gt;=B6),  --('Global GDP over time'!C6:C204&lt;=C6),  'Global GDP over time'!D6:D204 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A7:B118,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A7:B118,2,FALSE))</f>
+        <v>7401419828641</v>
+      </c>
+      <c r="M6" s="18">
         <f t="shared" si="3"/>
-        <v>0.02</v>
-      </c>
-      <c r="N6" s="5" t="s">
+        <v>0.05533333333</v>
+      </c>
+      <c r="N6" s="22">
+        <f>16.6/(3*100)</f>
+        <v>0.05533333333</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="P6" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="P6" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q6" s="14"/>
+      <c r="Q6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R6" s="14"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
@@ -1904,15 +1934,19 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="14"/>
-      <c r="P7" s="14"/>
+      <c r="L7" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C7:C205&gt;=B7),  --('Global GDP over time'!C7:C205&lt;=C7),  'Global GDP over time'!D7:D205 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A8:B119,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A8:B119,2,FALSE))</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="14"/>
       <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="8">
         <v>1968.0</v>
@@ -1938,35 +1972,41 @@
       </c>
       <c r="I8" s="6">
         <f>Constants!$B$1</f>
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="J8" s="15">
-        <f>L8*VLOOKUP(H8, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
-        <v>3525297429621</v>
+        <f>N8*VLOOKUP(H8, 'Global GDP over time'!$C$1:$E$49,3,TRUE)</f>
+        <v>1893326805386</v>
       </c>
       <c r="K8" s="15">
         <f>J8*(VLOOKUP(Constants!$B$1,'US CPI'!$A$2:$B$114,2,FALSE)/VLOOKUP(I8,'US CPI'!$A$2:$B$114,2,FALSE))</f>
-        <v>3525297429621</v>
-      </c>
-      <c r="L8" s="21">
-        <v>0.024</v>
-      </c>
-      <c r="M8" s="16">
-        <f>L8/D8</f>
-        <v>0.008</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="O8" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
+        <v>1893326805386</v>
+      </c>
+      <c r="L8" s="16">
+        <f>SUMPRODUCT(  --('Global GDP over time'!C8:C206&gt;=B8),  --('Global GDP over time'!C8:C206&lt;=C8),  'Global GDP over time'!D8:D206 ) * (VLOOKUP(Constants!$B$1,'US CPI'!A9:B120,2,FALSE) / VLOOKUP('Global GDP over time'!$I$4,'US CPI'!A9:B120,2,FALSE))</f>
+        <v>33607833537332</v>
+      </c>
+      <c r="M8" s="22">
+        <f>N8</f>
+        <v>0.012</v>
+      </c>
+      <c r="N8" s="22">
+        <v>0.012</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="P8" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q8" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R8" s="14"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -1979,22 +2019,23 @@
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
-      <c r="M9" s="16"/>
+      <c r="M9" s="18"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="14"/>
+      <c r="R9" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId4" ref="N2"/>
-    <hyperlink r:id="rId5" ref="O3"/>
-    <hyperlink r:id="rId6" ref="O4"/>
-    <hyperlink r:id="rId7" ref="N5"/>
-    <hyperlink r:id="rId8" ref="O5"/>
-    <hyperlink r:id="rId9" ref="O6"/>
-    <hyperlink r:id="rId10" ref="P6"/>
-    <hyperlink r:id="rId11" ref="O8"/>
+    <hyperlink r:id="rId4" ref="O2"/>
+    <hyperlink r:id="rId5" ref="P3"/>
+    <hyperlink r:id="rId6" ref="P4"/>
+    <hyperlink r:id="rId7" ref="O5"/>
+    <hyperlink r:id="rId8" ref="P5"/>
+    <hyperlink r:id="rId9" ref="P6"/>
+    <hyperlink r:id="rId10" ref="Q6"/>
+    <hyperlink r:id="rId11" ref="P8"/>
   </hyperlinks>
   <drawing r:id="rId12"/>
   <legacyDrawing r:id="rId13"/>
@@ -2013,902 +2054,902 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>58</v>
       </c>
+      <c r="B1" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>60</v>
+      </c>
       <c r="D1" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="E1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="26" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="27">
+      <c r="A2" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="28">
         <v>1.0</v>
       </c>
-      <c r="D2" s="28">
+      <c r="D2" s="29">
         <v>2.13E11</v>
       </c>
-      <c r="E2" s="29">
+      <c r="E2" s="16">
         <f>D2*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>254365973072</v>
+        <v>273223990208</v>
       </c>
       <c r="H2" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="B3" s="25" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="27">
+      <c r="C3" s="28">
         <v>1000.0</v>
       </c>
-      <c r="D3" s="28">
+      <c r="D3" s="29">
         <v>2.46E11</v>
       </c>
-      <c r="E3" s="29">
+      <c r="E3" s="16">
         <f>D3*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>293774785802</v>
+        <v>315554467564</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="27">
+      <c r="A4" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="28">
         <v>1500.0</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="29">
         <v>5.03E11</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="16">
         <f>D4*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>600685842513</v>
-      </c>
-      <c r="H4" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="I4" s="25">
+        <v>645219094247</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="I4" s="26">
         <v>2017.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="27">
+      <c r="A5" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="28">
         <v>1600.0</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="29">
         <v>6.71E11</v>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="16">
         <f>D5*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>801312525500</v>
+        <v>860719706242</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="27">
+      <c r="A6" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="28">
         <v>1700.0</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="29">
         <v>7.52E11</v>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="16">
         <f>D6*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>898043247654</v>
+        <v>964621787026</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="27">
+      <c r="A7" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="28">
         <v>1820.0</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="29">
         <v>1.4E12</v>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="16">
         <f>D7*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>1671889024888</v>
+        <v>1795838433293</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="27">
+      <c r="A8" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="28">
         <v>1850.0</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="29">
         <v>1.85E12</v>
       </c>
-      <c r="E8" s="29">
+      <c r="E8" s="16">
         <f>D8*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>2209281925745</v>
+        <v>2373072215422</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="27">
+      <c r="A9" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="28">
         <v>1870.0</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="29">
         <v>2.35E12</v>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="16">
         <f>D9*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>2806385148919</v>
+        <v>3014443084455</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="27">
+      <c r="A10" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="28">
         <v>1900.0</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="29">
         <v>4.19E12</v>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="16">
         <f>D10*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>5003725010200</v>
+        <v>5374687882497</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="27">
+      <c r="A11" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="28">
         <v>1920.0</v>
       </c>
-      <c r="D11" s="28">
+      <c r="D11" s="29">
         <v>5.77E12</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="16">
         <f>D11*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>6890571195430</v>
+        <v>7401419828641</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="27">
+      <c r="A12" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="28">
         <v>1940.0</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="29">
         <v>9.14E12</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="16">
         <f>D12*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>10915046919625</v>
+        <v>11724259485924</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="27">
+      <c r="A13" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="28">
         <v>1950.0</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="29">
         <v>1.01E13</v>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="16">
         <f>D13*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>12061485108119</v>
+        <v>12955691554468</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" s="27">
+      <c r="A14" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="28">
         <v>1960.0</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="29">
         <v>1.59E13</v>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="16">
         <f>D14*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>18987882496940</v>
+        <v>20395593635251</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="27">
+      <c r="A15" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="28">
         <v>1970.0</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="29">
         <v>2.62E13</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="16">
         <f>D15*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>31288208894329</v>
+        <v>33607833537332</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="27">
+      <c r="A16" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="28">
         <v>1980.0</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="29">
         <v>3.82E13</v>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="16">
         <f>D16*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>45618686250510</v>
+        <v>49000734394125</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="27">
+      <c r="A17" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="28">
         <v>1990.0</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="29">
         <v>5.14E13</v>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="16">
         <f>D17*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>61382211342309</v>
+        <v>65932925336597</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C18" s="27">
+      <c r="A18" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="28">
         <v>1991.0</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="29">
         <v>5.21E13</v>
       </c>
-      <c r="E18" s="29">
+      <c r="E18" s="16">
         <f>D18*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>62218155854753</v>
+        <v>66830844553244</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="27">
+      <c r="A19" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="28">
         <v>1992.0</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="29">
         <v>5.29E13</v>
       </c>
-      <c r="E19" s="29">
+      <c r="E19" s="16">
         <f>D19*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>63173521011832</v>
+        <v>67857037943697</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="27">
+      <c r="A20" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="28">
         <v>1993.0</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="29">
         <v>5.38E13</v>
       </c>
-      <c r="E20" s="29">
+      <c r="E20" s="16">
         <f>D20*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>64248306813546</v>
+        <v>69011505507956</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="27">
+      <c r="A21" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="28">
         <v>1994.0</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="29">
         <v>5.54E13</v>
       </c>
-      <c r="E21" s="29">
+      <c r="E21" s="16">
         <f>D21*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>66159037127703</v>
+        <v>71063892288862</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="27">
+      <c r="A22" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="28">
         <v>1995.0</v>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="29">
         <v>5.71E13</v>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="16">
         <f>D22*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>68189188086495</v>
+        <v>73244553243574</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="27">
+      <c r="A23" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="28">
         <v>1996.0</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="29">
         <v>5.92E13</v>
       </c>
-      <c r="E23" s="29">
+      <c r="E23" s="16">
         <f>D23*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>70697021623827</v>
+        <v>75938310893513</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24" s="27">
+      <c r="A24" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="28">
         <v>1997.0</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="29">
         <v>6.16E13</v>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="16">
         <f>D24*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>73563117095063</v>
+        <v>79016891064872</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C25" s="27">
+      <c r="A25" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="28">
         <v>1998.0</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="29">
         <v>6.31E13</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="16">
         <f>D25*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>75354426764586</v>
+        <v>80941003671971</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="27">
+      <c r="A26" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="28">
         <v>1999.0</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="29">
         <v>6.53E13</v>
       </c>
-      <c r="E26" s="29">
+      <c r="E26" s="16">
         <f>D26*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>77981680946552</v>
+        <v>83763035495716</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C27" s="27">
+      <c r="A27" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="28">
         <v>2000.0</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="29">
         <v>6.84E13</v>
       </c>
-      <c r="E27" s="29">
+      <c r="E27" s="16">
         <f>D27*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>81683720930233</v>
+        <v>87739534883721</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="27">
+      <c r="A28" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="28">
         <v>2001.0</v>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="29">
         <v>7.0E13</v>
       </c>
-      <c r="E28" s="29">
+      <c r="E28" s="16">
         <f>D28*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>83594451244390</v>
+        <v>89791921664627</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B29" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="27">
+      <c r="A29" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="28">
         <v>2002.0</v>
       </c>
-      <c r="D29" s="28">
+      <c r="D29" s="29">
         <v>7.19E13</v>
       </c>
-      <c r="E29" s="29">
+      <c r="E29" s="16">
         <f>D29*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>85863443492452</v>
+        <v>92229130966952</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B30" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C30" s="27">
+      <c r="A30" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="28">
         <v>2003.0</v>
       </c>
-      <c r="D30" s="28">
+      <c r="D30" s="29">
         <v>7.46E13</v>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="16">
         <f>D30*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>89087800897593</v>
+        <v>95692533659731</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="27">
+      <c r="A31" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="28">
         <v>2004.0</v>
       </c>
-      <c r="D31" s="28">
+      <c r="D31" s="29">
         <v>7.83E13</v>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="16">
         <f>D31*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>93506364749082</v>
+        <v>100438678090575</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="27">
+      <c r="A32" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="28">
         <v>2005.0</v>
       </c>
-      <c r="D32" s="28">
+      <c r="D32" s="29">
         <v>8.19E13</v>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="16">
         <f>D32*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>97805507955936</v>
+        <v>105056548347613</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C33" s="27">
+      <c r="A33" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="28">
         <v>2006.0</v>
       </c>
-      <c r="D33" s="28">
+      <c r="D33" s="29">
         <v>8.61E13</v>
       </c>
-      <c r="E33" s="29">
+      <c r="E33" s="16">
         <f>D33*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>102821175030600</v>
+        <v>110444063647491</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B34" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="27">
+      <c r="A34" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="28">
         <v>2007.0</v>
       </c>
-      <c r="D34" s="28">
+      <c r="D34" s="29">
         <v>9.05E13</v>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="16">
         <f>D34*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>108075683394533</v>
+        <v>116088127294982</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C35" s="27">
+      <c r="A35" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="28">
         <v>2008.0</v>
       </c>
-      <c r="D35" s="28">
+      <c r="D35" s="29">
         <v>9.29E13</v>
       </c>
-      <c r="E35" s="29">
+      <c r="E35" s="16">
         <f>D35*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>110941778865769</v>
+        <v>119166707466340</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B36" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="27">
+      <c r="A36" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="28">
         <v>2009.0</v>
       </c>
-      <c r="D36" s="28">
+      <c r="D36" s="29">
         <v>9.22E13</v>
       </c>
-      <c r="E36" s="29">
+      <c r="E36" s="16">
         <f>D36*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>110105834353325</v>
+        <v>118268788249694</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37" s="27">
+      <c r="A37" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="28">
         <v>2010.0</v>
       </c>
-      <c r="D37" s="28">
+      <c r="D37" s="29">
         <v>9.69E13</v>
       </c>
-      <c r="E37" s="29">
+      <c r="E37" s="16">
         <f>D37*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>115718604651163</v>
+        <v>124297674418605</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B38" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C38" s="27">
+      <c r="A38" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="28">
         <v>2011.0</v>
       </c>
-      <c r="D38" s="28">
+      <c r="D38" s="29">
         <v>1.01E14</v>
       </c>
-      <c r="E38" s="29">
+      <c r="E38" s="16">
         <f>D38*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>120614851081191</v>
+        <v>129556915544676</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B39" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C39" s="27">
+      <c r="A39" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="28">
         <v>2012.0</v>
       </c>
-      <c r="D39" s="28">
+      <c r="D39" s="29">
         <v>1.04E14</v>
       </c>
-      <c r="E39" s="29">
+      <c r="E39" s="16">
         <f>D39*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>124197470420237</v>
+        <v>133405140758874</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B40" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C40" s="27">
+      <c r="A40" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" s="28">
         <v>2013.0</v>
       </c>
-      <c r="D40" s="28">
+      <c r="D40" s="29">
         <v>1.07E14</v>
       </c>
-      <c r="E40" s="29">
+      <c r="E40" s="16">
         <f>D40*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>127780089759282</v>
+        <v>137253365973072</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B41" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="27">
+      <c r="A41" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B41" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="28">
         <v>2014.0</v>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="29">
         <v>1.11E14</v>
       </c>
-      <c r="E41" s="29">
+      <c r="E41" s="16">
         <f>D41*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>132556915544676</v>
+        <v>142384332925337</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B42" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C42" s="27">
+      <c r="A42" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" s="28">
         <v>2015.0</v>
       </c>
-      <c r="D42" s="28">
+      <c r="D42" s="29">
         <v>1.14E14</v>
       </c>
-      <c r="E42" s="29">
+      <c r="E42" s="16">
         <f>D42*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>136139534883721</v>
+        <v>146232558139535</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B43" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" s="27">
+      <c r="A43" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" s="28">
         <v>2016.0</v>
       </c>
-      <c r="D43" s="28">
+      <c r="D43" s="29">
         <v>1.18E14</v>
       </c>
-      <c r="E43" s="29">
+      <c r="E43" s="16">
         <f>D43*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>140916360669115</v>
+        <v>151363525091799</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B44" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C44" s="27">
+      <c r="A44" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B44" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C44" s="28">
         <v>2017.0</v>
       </c>
-      <c r="D44" s="28">
+      <c r="D44" s="29">
         <v>1.23E14</v>
       </c>
-      <c r="E44" s="29">
+      <c r="E44" s="16">
         <f>D44*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>146887392900857</v>
+        <v>157777233782130</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B45" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C45" s="27">
+      <c r="A45" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" s="28">
         <v>2018.0</v>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="29">
         <v>1.27E14</v>
       </c>
-      <c r="E45" s="29">
+      <c r="E45" s="16">
         <f>D45*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>151664218686251</v>
+        <v>162908200734394</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B46" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C46" s="27">
+      <c r="A46" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" s="28">
         <v>2019.0</v>
       </c>
-      <c r="D46" s="28">
+      <c r="D46" s="29">
         <v>1.31E14</v>
       </c>
-      <c r="E46" s="29">
+      <c r="E46" s="16">
         <f>D46*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>156441044471644</v>
+        <v>168039167686659</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B47" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C47" s="27">
+      <c r="A47" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" s="28">
         <v>2020.0</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="29">
         <v>1.27E14</v>
       </c>
-      <c r="E47" s="29">
+      <c r="E47" s="16">
         <f>D47*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>151664218686251</v>
+        <v>162908200734394</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B48" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" s="27">
+      <c r="A48" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="28">
         <v>2021.0</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="29">
         <v>1.35E14</v>
       </c>
-      <c r="E48" s="29">
+      <c r="E48" s="16">
         <f>D48*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>161217870257038</v>
+        <v>173170134638923</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B49" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C49" s="27">
+      <c r="A49" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C49" s="28">
         <v>2022.0</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="29">
         <v>1.39E14</v>
       </c>
-      <c r="E49" s="29">
+      <c r="E49" s="16">
         <f>D49*(VLOOKUP(Constants!$B$1,'US CPI'!$A$3:$B$114,2,FALSE)/VLOOKUP($I$4,'US CPI'!$A$3:$B$114,2,FALSE))</f>
-        <v>165994696042432</v>
+        <v>178301101591187</v>
       </c>
     </row>
   </sheetData>
@@ -2927,11 +2968,11 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" s="25">
-        <v>2022.0</v>
+      <c r="A1" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="26">
+        <v>2024.0</v>
       </c>
     </row>
   </sheetData>
@@ -2952,40 +2993,40 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E1" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>61</v>
+        <v>71</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" s="25" t="s">
+      <c r="A2" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>72</v>
       </c>
+      <c r="C2" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>74</v>
+      </c>
       <c r="I2" s="30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25">
+      <c r="A3" s="26">
         <v>1913.0</v>
       </c>
-      <c r="B3" s="25">
+      <c r="B3" s="26">
         <v>9.9</v>
       </c>
       <c r="E3" s="32">
@@ -2996,18 +3037,18 @@
         <f t="shared" ref="F3:F114" si="2">VLOOKUP(E3,$A$3:$B$114,2,FALSE)/VLOOKUP($J$3,$A$3:$B$114,2,FALSE)</f>
         <v>0.03148854962</v>
       </c>
-      <c r="I3" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="J3" s="25">
+      <c r="I3" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="26">
         <v>2024.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25">
+      <c r="A4" s="26">
         <v>1914.0</v>
       </c>
-      <c r="B4" s="25">
+      <c r="B4" s="26">
         <v>10.0</v>
       </c>
       <c r="C4" s="33">
@@ -3023,10 +3064,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25">
+      <c r="A5" s="26">
         <v>1915.0</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="26">
         <v>10.1</v>
       </c>
       <c r="C5" s="33">
@@ -3042,10 +3083,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25">
+      <c r="A6" s="26">
         <v>1916.0</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="26">
         <v>10.9</v>
       </c>
       <c r="C6" s="33">
@@ -3061,10 +3102,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25">
+      <c r="A7" s="26">
         <v>1917.0</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="26">
         <v>12.8</v>
       </c>
       <c r="C7" s="33">
@@ -3080,10 +3121,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25">
+      <c r="A8" s="26">
         <v>1918.0</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="26">
         <v>15.0</v>
       </c>
       <c r="C8" s="33">
@@ -3099,10 +3140,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25">
+      <c r="A9" s="26">
         <v>1919.0</v>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="26">
         <v>17.3</v>
       </c>
       <c r="C9" s="33">
@@ -3118,10 +3159,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25">
+      <c r="A10" s="26">
         <v>1920.0</v>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="26">
         <v>20.0</v>
       </c>
       <c r="C10" s="33">
@@ -3137,10 +3178,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25">
+      <c r="A11" s="26">
         <v>1921.0</v>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="26">
         <v>17.9</v>
       </c>
       <c r="C11" s="33">
@@ -3156,10 +3197,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25">
+      <c r="A12" s="26">
         <v>1922.0</v>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="26">
         <v>16.8</v>
       </c>
       <c r="C12" s="33">
@@ -3175,10 +3216,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25">
+      <c r="A13" s="26">
         <v>1923.0</v>
       </c>
-      <c r="B13" s="25">
+      <c r="B13" s="26">
         <v>17.1</v>
       </c>
       <c r="C13" s="33">
@@ -3194,10 +3235,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25">
+      <c r="A14" s="26">
         <v>1924.0</v>
       </c>
-      <c r="B14" s="25">
+      <c r="B14" s="26">
         <v>17.1</v>
       </c>
       <c r="C14" s="33">
@@ -3213,10 +3254,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25">
+      <c r="A15" s="26">
         <v>1925.0</v>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="26">
         <v>17.5</v>
       </c>
       <c r="C15" s="33">
@@ -3232,10 +3273,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25">
+      <c r="A16" s="26">
         <v>1926.0</v>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="26">
         <v>17.7</v>
       </c>
       <c r="C16" s="33">
@@ -3251,10 +3292,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25">
+      <c r="A17" s="26">
         <v>1927.0</v>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="26">
         <v>17.4</v>
       </c>
       <c r="C17" s="33">
@@ -3270,10 +3311,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25">
+      <c r="A18" s="26">
         <v>1928.0</v>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="26">
         <v>17.2</v>
       </c>
       <c r="C18" s="33">
@@ -3289,10 +3330,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25">
+      <c r="A19" s="26">
         <v>1929.0</v>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="26">
         <v>17.2</v>
       </c>
       <c r="C19" s="33">
@@ -3308,10 +3349,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25">
+      <c r="A20" s="26">
         <v>1930.0</v>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="26">
         <v>16.7</v>
       </c>
       <c r="C20" s="33">
@@ -3327,10 +3368,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25">
+      <c r="A21" s="26">
         <v>1931.0</v>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="26">
         <v>15.2</v>
       </c>
       <c r="C21" s="33">
@@ -3346,10 +3387,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25">
+      <c r="A22" s="26">
         <v>1932.0</v>
       </c>
-      <c r="B22" s="25">
+      <c r="B22" s="26">
         <v>13.6</v>
       </c>
       <c r="C22" s="33">
@@ -3365,10 +3406,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25">
+      <c r="A23" s="26">
         <v>1933.0</v>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="26">
         <v>12.9</v>
       </c>
       <c r="C23" s="33">
@@ -3384,10 +3425,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25">
+      <c r="A24" s="26">
         <v>1934.0</v>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="26">
         <v>13.4</v>
       </c>
       <c r="C24" s="33">
@@ -3403,10 +3444,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25">
+      <c r="A25" s="26">
         <v>1935.0</v>
       </c>
-      <c r="B25" s="25">
+      <c r="B25" s="26">
         <v>13.7</v>
       </c>
       <c r="C25" s="33">
@@ -3422,10 +3463,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25">
+      <c r="A26" s="26">
         <v>1936.0</v>
       </c>
-      <c r="B26" s="25">
+      <c r="B26" s="26">
         <v>13.9</v>
       </c>
       <c r="C26" s="33">
@@ -3441,10 +3482,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="25">
+      <c r="A27" s="26">
         <v>1937.0</v>
       </c>
-      <c r="B27" s="25">
+      <c r="B27" s="26">
         <v>14.4</v>
       </c>
       <c r="C27" s="33">
@@ -3460,10 +3501,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="25">
+      <c r="A28" s="26">
         <v>1938.0</v>
       </c>
-      <c r="B28" s="25">
+      <c r="B28" s="26">
         <v>14.1</v>
       </c>
       <c r="C28" s="33">
@@ -3479,10 +3520,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="25">
+      <c r="A29" s="26">
         <v>1939.0</v>
       </c>
-      <c r="B29" s="25">
+      <c r="B29" s="26">
         <v>13.9</v>
       </c>
       <c r="C29" s="33">
@@ -3498,10 +3539,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="25">
+      <c r="A30" s="26">
         <v>1940.0</v>
       </c>
-      <c r="B30" s="25">
+      <c r="B30" s="26">
         <v>14.0</v>
       </c>
       <c r="C30" s="33">
@@ -3517,10 +3558,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25">
+      <c r="A31" s="26">
         <v>1941.0</v>
       </c>
-      <c r="B31" s="25">
+      <c r="B31" s="26">
         <v>14.7</v>
       </c>
       <c r="C31" s="33">
@@ -3536,10 +3577,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="25">
+      <c r="A32" s="26">
         <v>1942.0</v>
       </c>
-      <c r="B32" s="25">
+      <c r="B32" s="26">
         <v>16.3</v>
       </c>
       <c r="C32" s="33">
@@ -3555,10 +3596,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="25">
+      <c r="A33" s="26">
         <v>1943.0</v>
       </c>
-      <c r="B33" s="25">
+      <c r="B33" s="26">
         <v>17.3</v>
       </c>
       <c r="C33" s="33">
@@ -3574,10 +3615,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="25">
+      <c r="A34" s="26">
         <v>1944.0</v>
       </c>
-      <c r="B34" s="25">
+      <c r="B34" s="26">
         <v>17.6</v>
       </c>
       <c r="C34" s="33">
@@ -3593,10 +3634,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="25">
+      <c r="A35" s="26">
         <v>1945.0</v>
       </c>
-      <c r="B35" s="25">
+      <c r="B35" s="26">
         <v>18.0</v>
       </c>
       <c r="C35" s="33">
@@ -3612,10 +3653,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="25">
+      <c r="A36" s="26">
         <v>1946.0</v>
       </c>
-      <c r="B36" s="25">
+      <c r="B36" s="26">
         <v>19.5</v>
       </c>
       <c r="C36" s="33">
@@ -3631,10 +3672,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="25">
+      <c r="A37" s="26">
         <v>1947.0</v>
       </c>
-      <c r="B37" s="25">
+      <c r="B37" s="26">
         <v>22.3</v>
       </c>
       <c r="C37" s="33">
@@ -3650,10 +3691,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="25">
+      <c r="A38" s="26">
         <v>1948.0</v>
       </c>
-      <c r="B38" s="25">
+      <c r="B38" s="26">
         <v>24.0</v>
       </c>
       <c r="C38" s="33">
@@ -3669,10 +3710,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="25">
+      <c r="A39" s="26">
         <v>1949.0</v>
       </c>
-      <c r="B39" s="25">
+      <c r="B39" s="26">
         <v>23.8</v>
       </c>
       <c r="C39" s="33">
@@ -3688,10 +3729,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="25">
+      <c r="A40" s="26">
         <v>1950.0</v>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="26">
         <v>24.1</v>
       </c>
       <c r="C40" s="33">
@@ -3707,10 +3748,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="25">
+      <c r="A41" s="26">
         <v>1951.0</v>
       </c>
-      <c r="B41" s="25">
+      <c r="B41" s="26">
         <v>26.0</v>
       </c>
       <c r="C41" s="33">
@@ -3726,10 +3767,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="25">
+      <c r="A42" s="26">
         <v>1952.0</v>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="26">
         <v>26.6</v>
       </c>
       <c r="C42" s="33">
@@ -3745,10 +3786,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25">
+      <c r="A43" s="26">
         <v>1953.0</v>
       </c>
-      <c r="B43" s="25">
+      <c r="B43" s="26">
         <v>26.8</v>
       </c>
       <c r="C43" s="33">
@@ -3764,10 +3805,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="25">
+      <c r="A44" s="26">
         <v>1954.0</v>
       </c>
-      <c r="B44" s="25">
+      <c r="B44" s="26">
         <v>26.9</v>
       </c>
       <c r="C44" s="33">
@@ -3783,10 +3824,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="25">
+      <c r="A45" s="26">
         <v>1955.0</v>
       </c>
-      <c r="B45" s="25">
+      <c r="B45" s="26">
         <v>26.8</v>
       </c>
       <c r="C45" s="33">
@@ -3802,10 +3843,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="25">
+      <c r="A46" s="26">
         <v>1956.0</v>
       </c>
-      <c r="B46" s="25">
+      <c r="B46" s="26">
         <v>27.2</v>
       </c>
       <c r="C46" s="33">
@@ -3821,10 +3862,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25">
+      <c r="A47" s="26">
         <v>1957.0</v>
       </c>
-      <c r="B47" s="25">
+      <c r="B47" s="26">
         <v>28.1</v>
       </c>
       <c r="C47" s="33">
@@ -3840,10 +3881,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25">
+      <c r="A48" s="26">
         <v>1958.0</v>
       </c>
-      <c r="B48" s="25">
+      <c r="B48" s="26">
         <v>28.9</v>
       </c>
       <c r="C48" s="33">
@@ -3859,10 +3900,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="25">
+      <c r="A49" s="26">
         <v>1959.0</v>
       </c>
-      <c r="B49" s="25">
+      <c r="B49" s="26">
         <v>29.2</v>
       </c>
       <c r="C49" s="33">
@@ -3878,10 +3919,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="25">
+      <c r="A50" s="26">
         <v>1960.0</v>
       </c>
-      <c r="B50" s="25">
+      <c r="B50" s="26">
         <v>29.6</v>
       </c>
       <c r="C50" s="33">
@@ -3897,10 +3938,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="25">
+      <c r="A51" s="26">
         <v>1961.0</v>
       </c>
-      <c r="B51" s="25">
+      <c r="B51" s="26">
         <v>29.9</v>
       </c>
       <c r="C51" s="33">
@@ -3916,10 +3957,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25">
+      <c r="A52" s="26">
         <v>1962.0</v>
       </c>
-      <c r="B52" s="25">
+      <c r="B52" s="26">
         <v>30.3</v>
       </c>
       <c r="C52" s="33">
@@ -3935,10 +3976,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="25">
+      <c r="A53" s="26">
         <v>1963.0</v>
       </c>
-      <c r="B53" s="25">
+      <c r="B53" s="26">
         <v>30.6</v>
       </c>
       <c r="C53" s="33">
@@ -3954,10 +3995,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="25">
+      <c r="A54" s="26">
         <v>1964.0</v>
       </c>
-      <c r="B54" s="25">
+      <c r="B54" s="26">
         <v>31.0</v>
       </c>
       <c r="C54" s="33">
@@ -3973,10 +4014,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="25">
+      <c r="A55" s="26">
         <v>1965.0</v>
       </c>
-      <c r="B55" s="25">
+      <c r="B55" s="26">
         <v>31.5</v>
       </c>
       <c r="C55" s="33">
@@ -3992,10 +4033,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="25">
+      <c r="A56" s="26">
         <v>1966.0</v>
       </c>
-      <c r="B56" s="25">
+      <c r="B56" s="26">
         <v>32.5</v>
       </c>
       <c r="C56" s="33">
@@ -4011,10 +4052,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="25">
+      <c r="A57" s="26">
         <v>1967.0</v>
       </c>
-      <c r="B57" s="25">
+      <c r="B57" s="26">
         <v>33.4</v>
       </c>
       <c r="C57" s="33">
@@ -4030,10 +4071,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="25">
+      <c r="A58" s="26">
         <v>1968.0</v>
       </c>
-      <c r="B58" s="25">
+      <c r="B58" s="26">
         <v>34.8</v>
       </c>
       <c r="C58" s="33">
@@ -4049,10 +4090,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25">
+      <c r="A59" s="26">
         <v>1969.0</v>
       </c>
-      <c r="B59" s="25">
+      <c r="B59" s="26">
         <v>36.7</v>
       </c>
       <c r="C59" s="33">
@@ -4068,10 +4109,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="25">
+      <c r="A60" s="26">
         <v>1970.0</v>
       </c>
-      <c r="B60" s="25">
+      <c r="B60" s="26">
         <v>38.8</v>
       </c>
       <c r="C60" s="33">
@@ -4087,10 +4128,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="25">
+      <c r="A61" s="26">
         <v>1971.0</v>
       </c>
-      <c r="B61" s="25">
+      <c r="B61" s="26">
         <v>40.5</v>
       </c>
       <c r="C61" s="33">
@@ -4106,10 +4147,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="25">
+      <c r="A62" s="26">
         <v>1972.0</v>
       </c>
-      <c r="B62" s="25">
+      <c r="B62" s="26">
         <v>41.8</v>
       </c>
       <c r="C62" s="33">
@@ -4125,10 +4166,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="25">
+      <c r="A63" s="26">
         <v>1973.0</v>
       </c>
-      <c r="B63" s="25">
+      <c r="B63" s="26">
         <v>44.4</v>
       </c>
       <c r="C63" s="33">
@@ -4144,10 +4185,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="25">
+      <c r="A64" s="26">
         <v>1974.0</v>
       </c>
-      <c r="B64" s="25">
+      <c r="B64" s="26">
         <v>49.3</v>
       </c>
       <c r="C64" s="33">
@@ -4163,10 +4204,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="25">
+      <c r="A65" s="26">
         <v>1975.0</v>
       </c>
-      <c r="B65" s="25">
+      <c r="B65" s="26">
         <v>53.8</v>
       </c>
       <c r="C65" s="33">
@@ -4182,10 +4223,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="25">
+      <c r="A66" s="26">
         <v>1976.0</v>
       </c>
-      <c r="B66" s="25">
+      <c r="B66" s="26">
         <v>56.9</v>
       </c>
       <c r="C66" s="33">
@@ -4201,10 +4242,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="25">
+      <c r="A67" s="26">
         <v>1977.0</v>
       </c>
-      <c r="B67" s="25">
+      <c r="B67" s="26">
         <v>60.6</v>
       </c>
       <c r="C67" s="33">
@@ -4220,10 +4261,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="25">
+      <c r="A68" s="26">
         <v>1978.0</v>
       </c>
-      <c r="B68" s="25">
+      <c r="B68" s="26">
         <v>65.2</v>
       </c>
       <c r="C68" s="33">
@@ -4239,10 +4280,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="25">
+      <c r="A69" s="26">
         <v>1979.0</v>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="26">
         <v>72.6</v>
       </c>
       <c r="C69" s="33">
@@ -4258,10 +4299,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="25">
+      <c r="A70" s="26">
         <v>1980.0</v>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="26">
         <v>82.4</v>
       </c>
       <c r="C70" s="33">
@@ -4277,10 +4318,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="25">
+      <c r="A71" s="26">
         <v>1981.0</v>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="26">
         <v>90.9</v>
       </c>
       <c r="C71" s="33">
@@ -4296,10 +4337,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="25">
+      <c r="A72" s="26">
         <v>1982.0</v>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="26">
         <v>96.5</v>
       </c>
       <c r="C72" s="33">
@@ -4315,10 +4356,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="25">
+      <c r="A73" s="26">
         <v>1983.0</v>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="26">
         <v>99.6</v>
       </c>
       <c r="C73" s="33">
@@ -4334,10 +4375,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="25">
+      <c r="A74" s="26">
         <v>1984.0</v>
       </c>
-      <c r="B74" s="25">
+      <c r="B74" s="26">
         <v>103.9</v>
       </c>
       <c r="C74" s="33">
@@ -4353,10 +4394,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="25">
+      <c r="A75" s="26">
         <v>1985.0</v>
       </c>
-      <c r="B75" s="25">
+      <c r="B75" s="26">
         <v>107.6</v>
       </c>
       <c r="C75" s="33">
@@ -4372,10 +4413,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="25">
+      <c r="A76" s="26">
         <v>1986.0</v>
       </c>
-      <c r="B76" s="25">
+      <c r="B76" s="26">
         <v>109.6</v>
       </c>
       <c r="C76" s="33">
@@ -4391,10 +4432,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="25">
+      <c r="A77" s="26">
         <v>1987.0</v>
       </c>
-      <c r="B77" s="25">
+      <c r="B77" s="26">
         <v>113.6</v>
       </c>
       <c r="C77" s="33">
@@ -4410,10 +4451,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="25">
+      <c r="A78" s="26">
         <v>1988.0</v>
       </c>
-      <c r="B78" s="25">
+      <c r="B78" s="26">
         <v>118.3</v>
       </c>
       <c r="C78" s="33">
@@ -4429,10 +4470,10 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="25">
+      <c r="A79" s="26">
         <v>1989.0</v>
       </c>
-      <c r="B79" s="25">
+      <c r="B79" s="26">
         <v>124.0</v>
       </c>
       <c r="C79" s="33">
@@ -4448,10 +4489,10 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="25">
+      <c r="A80" s="26">
         <v>1990.0</v>
       </c>
-      <c r="B80" s="25">
+      <c r="B80" s="26">
         <v>130.7</v>
       </c>
       <c r="C80" s="33">
@@ -4467,10 +4508,10 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="25">
+      <c r="A81" s="26">
         <v>1991.0</v>
       </c>
-      <c r="B81" s="25">
+      <c r="B81" s="26">
         <v>136.2</v>
       </c>
       <c r="C81" s="33">
@@ -4486,10 +4527,10 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="25">
+      <c r="A82" s="26">
         <v>1992.0</v>
       </c>
-      <c r="B82" s="25">
+      <c r="B82" s="26">
         <v>140.3</v>
       </c>
       <c r="C82" s="33">
@@ -4505,10 +4546,10 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="25">
+      <c r="A83" s="26">
         <v>1993.0</v>
       </c>
-      <c r="B83" s="25">
+      <c r="B83" s="26">
         <v>144.5</v>
       </c>
       <c r="C83" s="33">
@@ -4524,10 +4565,10 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="25">
+      <c r="A84" s="26">
         <v>1994.0</v>
       </c>
-      <c r="B84" s="25">
+      <c r="B84" s="26">
         <v>148.2</v>
       </c>
       <c r="C84" s="33">
@@ -4543,10 +4584,10 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="25">
+      <c r="A85" s="26">
         <v>1995.0</v>
       </c>
-      <c r="B85" s="25">
+      <c r="B85" s="26">
         <v>152.4</v>
       </c>
       <c r="C85" s="33">
@@ -4562,10 +4603,10 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="25">
+      <c r="A86" s="26">
         <v>1996.0</v>
       </c>
-      <c r="B86" s="25">
+      <c r="B86" s="26">
         <v>156.9</v>
       </c>
       <c r="C86" s="33">
@@ -4581,10 +4622,10 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="25">
+      <c r="A87" s="26">
         <v>1997.0</v>
       </c>
-      <c r="B87" s="25">
+      <c r="B87" s="26">
         <v>160.5</v>
       </c>
       <c r="C87" s="33">
@@ -4600,10 +4641,10 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="25">
+      <c r="A88" s="26">
         <v>1998.0</v>
       </c>
-      <c r="B88" s="25">
+      <c r="B88" s="26">
         <v>163.0</v>
       </c>
       <c r="C88" s="33">
@@ -4619,10 +4660,10 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="25">
+      <c r="A89" s="26">
         <v>1999.0</v>
       </c>
-      <c r="B89" s="25">
+      <c r="B89" s="26">
         <v>166.6</v>
       </c>
       <c r="C89" s="33">
@@ -4638,10 +4679,10 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="25">
+      <c r="A90" s="26">
         <v>2000.0</v>
       </c>
-      <c r="B90" s="25">
+      <c r="B90" s="26">
         <v>172.2</v>
       </c>
       <c r="C90" s="33">
@@ -4657,10 +4698,10 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="25">
+      <c r="A91" s="26">
         <v>2001.0</v>
       </c>
-      <c r="B91" s="25">
+      <c r="B91" s="26">
         <v>177.1</v>
       </c>
       <c r="C91" s="33">
@@ -4676,10 +4717,10 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="25">
+      <c r="A92" s="26">
         <v>2002.0</v>
       </c>
-      <c r="B92" s="25">
+      <c r="B92" s="26">
         <v>179.9</v>
       </c>
       <c r="C92" s="33">
@@ -4695,10 +4736,10 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="25">
+      <c r="A93" s="26">
         <v>2003.0</v>
       </c>
-      <c r="B93" s="25">
+      <c r="B93" s="26">
         <v>184.0</v>
       </c>
       <c r="C93" s="33">
@@ -4714,10 +4755,10 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="25">
+      <c r="A94" s="26">
         <v>2004.0</v>
       </c>
-      <c r="B94" s="25">
+      <c r="B94" s="26">
         <v>188.9</v>
       </c>
       <c r="C94" s="33">
@@ -4733,10 +4774,10 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="25">
+      <c r="A95" s="26">
         <v>2005.0</v>
       </c>
-      <c r="B95" s="25">
+      <c r="B95" s="26">
         <v>195.3</v>
       </c>
       <c r="C95" s="33">
@@ -4752,10 +4793,10 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="25">
+      <c r="A96" s="26">
         <v>2006.0</v>
       </c>
-      <c r="B96" s="25">
+      <c r="B96" s="26">
         <v>201.6</v>
       </c>
       <c r="C96" s="33">
@@ -4771,10 +4812,10 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="25">
+      <c r="A97" s="26">
         <v>2007.0</v>
       </c>
-      <c r="B97" s="25">
+      <c r="B97" s="26">
         <v>207.3</v>
       </c>
       <c r="C97" s="33">
@@ -4790,10 +4831,10 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="25">
+      <c r="A98" s="26">
         <v>2008.0</v>
       </c>
-      <c r="B98" s="25">
+      <c r="B98" s="26">
         <v>215.3</v>
       </c>
       <c r="C98" s="33">
@@ -4809,10 +4850,10 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="25">
+      <c r="A99" s="26">
         <v>2009.0</v>
       </c>
-      <c r="B99" s="25">
+      <c r="B99" s="26">
         <v>214.5</v>
       </c>
       <c r="C99" s="33">
@@ -4828,10 +4869,10 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="25">
+      <c r="A100" s="26">
         <v>2010.0</v>
       </c>
-      <c r="B100" s="25">
+      <c r="B100" s="26">
         <v>218.1</v>
       </c>
       <c r="C100" s="33">
@@ -4847,10 +4888,10 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="25">
+      <c r="A101" s="26">
         <v>2011.0</v>
       </c>
-      <c r="B101" s="25">
+      <c r="B101" s="26">
         <v>224.9</v>
       </c>
       <c r="C101" s="33">
@@ -4866,10 +4907,10 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="25">
+      <c r="A102" s="26">
         <v>2012.0</v>
       </c>
-      <c r="B102" s="25">
+      <c r="B102" s="26">
         <v>229.6</v>
       </c>
       <c r="C102" s="33">
@@ -4885,10 +4926,10 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="25">
+      <c r="A103" s="26">
         <v>2013.0</v>
       </c>
-      <c r="B103" s="25">
+      <c r="B103" s="26">
         <v>233.0</v>
       </c>
       <c r="C103" s="33">
@@ -4904,10 +4945,10 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="25">
+      <c r="A104" s="26">
         <v>2014.0</v>
       </c>
-      <c r="B104" s="25">
+      <c r="B104" s="26">
         <v>236.7</v>
       </c>
       <c r="C104" s="33">
@@ -4923,10 +4964,10 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="25">
+      <c r="A105" s="26">
         <v>2015.0</v>
       </c>
-      <c r="B105" s="25">
+      <c r="B105" s="26">
         <v>237.0</v>
       </c>
       <c r="C105" s="33">
@@ -4942,10 +4983,10 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="25">
+      <c r="A106" s="26">
         <v>2016.0</v>
       </c>
-      <c r="B106" s="25">
+      <c r="B106" s="26">
         <v>240.0</v>
       </c>
       <c r="C106" s="33">
@@ -4961,10 +5002,10 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="25">
+      <c r="A107" s="26">
         <v>2017.0</v>
       </c>
-      <c r="B107" s="25">
+      <c r="B107" s="26">
         <v>245.1</v>
       </c>
       <c r="C107" s="33">
@@ -4980,10 +5021,10 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="25">
+      <c r="A108" s="26">
         <v>2018.0</v>
       </c>
-      <c r="B108" s="25">
+      <c r="B108" s="26">
         <v>251.1</v>
       </c>
       <c r="C108" s="33">
@@ -4999,10 +5040,10 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="25">
+      <c r="A109" s="26">
         <v>2019.0</v>
       </c>
-      <c r="B109" s="25">
+      <c r="B109" s="26">
         <v>255.7</v>
       </c>
       <c r="C109" s="33">
@@ -5018,10 +5059,10 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="25">
+      <c r="A110" s="26">
         <v>2020.0</v>
       </c>
-      <c r="B110" s="25">
+      <c r="B110" s="26">
         <v>258.8</v>
       </c>
       <c r="C110" s="33">
@@ -5037,10 +5078,10 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="25">
+      <c r="A111" s="26">
         <v>2021.0</v>
       </c>
-      <c r="B111" s="25">
+      <c r="B111" s="26">
         <v>271.0</v>
       </c>
       <c r="C111" s="33">
@@ -5056,10 +5097,10 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="25">
+      <c r="A112" s="26">
         <v>2022.0</v>
       </c>
-      <c r="B112" s="25">
+      <c r="B112" s="26">
         <v>292.7</v>
       </c>
       <c r="C112" s="33">
@@ -5075,10 +5116,10 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="25">
+      <c r="A113" s="26">
         <v>2023.0</v>
       </c>
-      <c r="B113" s="25">
+      <c r="B113" s="26">
         <v>304.7</v>
       </c>
       <c r="C113" s="33">
@@ -5094,10 +5135,10 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="25">
+      <c r="A114" s="26">
         <v>2024.0</v>
       </c>
-      <c r="B114" s="25">
+      <c r="B114" s="26">
         <v>314.4</v>
       </c>
       <c r="C114" s="33">

</xml_diff>